<commit_message>
NSP P8/09: record owner manual Excel acceptance and promote exact reviewed bytes [skip deploy]
</commit_message>
<xml_diff>
--- a/products-storage/10-avans-usloviya-i-pribyl/09-raschet-otrabotannoy-chasti-avansa.xlsx
+++ b/products-storage/10-avans-usloviya-i-pribyl/09-raschet-otrabotannoy-chasti-avansa.xlsx
@@ -670,7 +670,7 @@
     <row r="12" ht="33" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2. На листе «Выполнено» зарегистрируйте все акты, отдельно указав статус подписания, дату передачи и её подтверждение.</t>
+          <t>2. Заполните документ, номер, стоимость и статус каждого акта. Оплаты и погашение аванса укажите числами; отсутствие — 0. Для неподписанных актов подтвердите передачу.</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <row r="14" ht="33" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">4. На листе «Сальдо» проверьте исходные данные и сообщения контроля, затем сопоставьте итог с требованием о возврате.</t>
+          <t>4. Исправьте строки «ОШИБКА» и «НЕ ЗАПОЛНЕНО». При неполных данных итог сальдо и итоговая запись акта сверки не выводятся.</t>
         </is>
       </c>
     </row>
@@ -719,7 +719,7 @@
     <row r="19" ht="19" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>До подписания сверки проверьте встречные расчёты, аванс и все акты.</t>
+          <t>Частичная денежная оплата уменьшает остаток каждого акта. Отсутствие подписи не меняется от оплаты; правовое основание требования проверьте отдельно.</t>
         </is>
       </c>
     </row>
@@ -953,7 +953,7 @@
         </is>
       </c>
       <c r="B17" s="8">
-        <f>MAX(0,B6-B16)</f>
+        <f>IF(OR(NOT(ISNUMBER(B6)),NOT(ISNUMBER(B16))),"",MAX(0,B6-B16))</f>
         <v/>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="B19" s="11">
-        <f>IF(B5="","не заполнена цена договора",IF(B6="","не заполнена сумма полученного аванса",IF(B8="","не выбрано основание прекращения договора",IF(B11="","не заполнена сумма требования",IF(B6&gt;B5,"ПРОВЕРЬТЕ: аванс больше цены договора","заполнено")))))</f>
+        <f>IF(OR(LEN(B5)=0,LEN(B6)=0,LEN(B8)=0,LEN(B11)=0),"НЕ ЗАПОЛНЕНО: цена, аванс, основание и сумма требования",IF(OR(NOT(ISNUMBER(B5)),NOT(ISNUMBER(B6)),NOT(ISNUMBER(B11))),"ОШИБКА: суммы договора должны быть числами",IF(OR(B5&lt;=0,B6&lt;0,B11&lt;0),"ОШИБКА: проверьте знак и величину сумм",IF(COUNTIF($A$22:$A$27,B8)&lt;&gt;1,"ОШИБКА: выберите основание из справочника",IF(B6&gt;B5,"ПРОВЕРЬТЕ: аванс больше цены договора","заполнено")))))</f>
         <v/>
       </c>
       <c r="C19" s="12" t="n"/>
@@ -1055,8 +1055,8 @@
     <mergeCell ref="A15:C15"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="B8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Выберите основание из списка" type="list">
-      <formula1>=$A$22:$A$27</formula1>
+    <dataValidation type="list" errorStyle="stop" allowBlank="0" showDropDown="0" showErrorMessage="1" errorTitle="Проверка ввода" error="Выберите основание из справочника." sqref="B8">
+      <formula1>$A$22:$A$27</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1073,7 +1073,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:N57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1088,6 +1088,7 @@
     <col width="15" customWidth="1" min="10" max="10"/>
     <col width="15" customWidth="1" min="11" max="11"/>
     <col width="34" customWidth="1" min="12" max="12"/>
+    <col min="14" max="14" width="48" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1096,11 +1097,35 @@
           <t xml:space="preserve">Реестр актов выполненных работ</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Справочник статусов актов</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>подписан обеими сторонами</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="44" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Зарегистрируйте все акты по объекту. Для каждого укажите статус подписания, дату передачи и подтверждающий документ. Раздельный учёт двусторонних и односторонних актов необходим для сверки признанных и спорных сумм.</t>
+          <t>Запишите документ, номер, стоимость и выберите статус из списка. Погашение аванса и денежную оплату укажите числами; при отсутствии — 0. Для неподписанных и односторонних актов нужны дата и подтверждение передачи.</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>передан, не подписан</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>подписан односторонне</t>
         </is>
       </c>
     </row>
@@ -1163,6 +1188,11 @@
       <c r="L5" s="14" t="inlineStr">
         <is>
           <t>Проверка</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>получен мотивированный отказ</t>
         </is>
       </c>
     </row>
@@ -1181,11 +1211,12 @@
       <c r="I6" s="17" t="n"/>
       <c r="J6" s="17" t="n"/>
       <c r="K6" s="19">
-        <f>IF(E6="","",ROUND(E6-I6-J6,2))</f>
+        <f>IF(L6="строка заполнена",ROUND(E6-I6-J6,2),"")</f>
         <v/>
       </c>
       <c r="L6" s="15">
-        <f>IF(E6="","",IF(F6="","не выбран статус",IF(I6+J6&gt;E6+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F6&lt;&gt;"подписан обеими сторонами",I6&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F6="подписан обеими сторонами",I6+J6=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F6&lt;&gt;"подписан обеими сторонами",G6=""),"Акт не подписан: укажите дату передачи.",IF(AND(F6&lt;&gt;"подписан обеими сторонами",H6=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B6:J6)=0,"",IF(OR(LEN(B6)=0,LEN(C6)=0,LEN(E6)=0,LEN(F6)=0,LEN(I6)=0,LEN(J6)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F6)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E6)),NOT(ISNUMBER(I6)),NOT(ISNUMBER(J6))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E6&lt;0,I6&lt;0,J6&lt;0),"ОШИБКА: отрицательная сумма",IF(I6+J6&gt;E6+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F6&lt;&gt;"подписан обеими сторонами",I6&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F6&lt;&gt;"подписан обеими сторонами",OR(LEN(G6)=0,LEN(H6)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F6&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G6)),G6&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
@@ -1203,11 +1234,12 @@
       <c r="I7" s="17" t="n"/>
       <c r="J7" s="17" t="n"/>
       <c r="K7" s="19">
-        <f>IF(E7="","",ROUND(E7-I7-J7,2))</f>
+        <f>IF(L7="строка заполнена",ROUND(E7-I7-J7,2),"")</f>
         <v/>
       </c>
       <c r="L7" s="15">
-        <f>IF(E7="","",IF(F7="","не выбран статус",IF(I7+J7&gt;E7+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F7&lt;&gt;"подписан обеими сторонами",I7&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F7="подписан обеими сторонами",I7+J7=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F7&lt;&gt;"подписан обеими сторонами",G7=""),"Акт не подписан: укажите дату передачи.",IF(AND(F7&lt;&gt;"подписан обеими сторонами",H7=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B7:J7)=0,"",IF(OR(LEN(B7)=0,LEN(C7)=0,LEN(E7)=0,LEN(F7)=0,LEN(I7)=0,LEN(J7)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F7)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E7)),NOT(ISNUMBER(I7)),NOT(ISNUMBER(J7))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E7&lt;0,I7&lt;0,J7&lt;0),"ОШИБКА: отрицательная сумма",IF(I7+J7&gt;E7+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F7&lt;&gt;"подписан обеими сторонами",I7&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F7&lt;&gt;"подписан обеими сторонами",OR(LEN(G7)=0,LEN(H7)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F7&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G7)),G7&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1">
@@ -1225,11 +1257,12 @@
       <c r="I8" s="17" t="n"/>
       <c r="J8" s="17" t="n"/>
       <c r="K8" s="19">
-        <f>IF(E8="","",ROUND(E8-I8-J8,2))</f>
+        <f>IF(L8="строка заполнена",ROUND(E8-I8-J8,2),"")</f>
         <v/>
       </c>
       <c r="L8" s="15">
-        <f>IF(E8="","",IF(F8="","не выбран статус",IF(I8+J8&gt;E8+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F8&lt;&gt;"подписан обеими сторонами",I8&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F8="подписан обеими сторонами",I8+J8=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F8&lt;&gt;"подписан обеими сторонами",G8=""),"Акт не подписан: укажите дату передачи.",IF(AND(F8&lt;&gt;"подписан обеими сторонами",H8=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B8:J8)=0,"",IF(OR(LEN(B8)=0,LEN(C8)=0,LEN(E8)=0,LEN(F8)=0,LEN(I8)=0,LEN(J8)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F8)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E8)),NOT(ISNUMBER(I8)),NOT(ISNUMBER(J8))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E8&lt;0,I8&lt;0,J8&lt;0),"ОШИБКА: отрицательная сумма",IF(I8+J8&gt;E8+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F8&lt;&gt;"подписан обеими сторонами",I8&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F8&lt;&gt;"подписан обеими сторонами",OR(LEN(G8)=0,LEN(H8)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F8&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G8)),G8&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
@@ -1247,11 +1280,12 @@
       <c r="I9" s="17" t="n"/>
       <c r="J9" s="17" t="n"/>
       <c r="K9" s="19">
-        <f>IF(E9="","",ROUND(E9-I9-J9,2))</f>
+        <f>IF(L9="строка заполнена",ROUND(E9-I9-J9,2),"")</f>
         <v/>
       </c>
       <c r="L9" s="15">
-        <f>IF(E9="","",IF(F9="","не выбран статус",IF(I9+J9&gt;E9+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F9&lt;&gt;"подписан обеими сторонами",I9&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F9="подписан обеими сторонами",I9+J9=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F9&lt;&gt;"подписан обеими сторонами",G9=""),"Акт не подписан: укажите дату передачи.",IF(AND(F9&lt;&gt;"подписан обеими сторонами",H9=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B9:J9)=0,"",IF(OR(LEN(B9)=0,LEN(C9)=0,LEN(E9)=0,LEN(F9)=0,LEN(I9)=0,LEN(J9)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F9)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E9)),NOT(ISNUMBER(I9)),NOT(ISNUMBER(J9))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E9&lt;0,I9&lt;0,J9&lt;0),"ОШИБКА: отрицательная сумма",IF(I9+J9&gt;E9+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F9&lt;&gt;"подписан обеими сторонами",I9&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F9&lt;&gt;"подписан обеими сторонами",OR(LEN(G9)=0,LEN(H9)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F9&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G9)),G9&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">
@@ -1269,11 +1303,12 @@
       <c r="I10" s="17" t="n"/>
       <c r="J10" s="17" t="n"/>
       <c r="K10" s="19">
-        <f>IF(E10="","",ROUND(E10-I10-J10,2))</f>
+        <f>IF(L10="строка заполнена",ROUND(E10-I10-J10,2),"")</f>
         <v/>
       </c>
       <c r="L10" s="15">
-        <f>IF(E10="","",IF(F10="","не выбран статус",IF(I10+J10&gt;E10+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F10&lt;&gt;"подписан обеими сторонами",I10&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F10="подписан обеими сторонами",I10+J10=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F10&lt;&gt;"подписан обеими сторонами",G10=""),"Акт не подписан: укажите дату передачи.",IF(AND(F10&lt;&gt;"подписан обеими сторонами",H10=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B10:J10)=0,"",IF(OR(LEN(B10)=0,LEN(C10)=0,LEN(E10)=0,LEN(F10)=0,LEN(I10)=0,LEN(J10)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F10)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E10)),NOT(ISNUMBER(I10)),NOT(ISNUMBER(J10))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E10&lt;0,I10&lt;0,J10&lt;0),"ОШИБКА: отрицательная сумма",IF(I10+J10&gt;E10+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F10&lt;&gt;"подписан обеими сторонами",I10&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F10&lt;&gt;"подписан обеими сторонами",OR(LEN(G10)=0,LEN(H10)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F10&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G10)),G10&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="11" ht="45" customHeight="1">
@@ -1291,11 +1326,12 @@
       <c r="I11" s="17" t="n"/>
       <c r="J11" s="17" t="n"/>
       <c r="K11" s="19">
-        <f>IF(E11="","",ROUND(E11-I11-J11,2))</f>
+        <f>IF(L11="строка заполнена",ROUND(E11-I11-J11,2),"")</f>
         <v/>
       </c>
       <c r="L11" s="15">
-        <f>IF(E11="","",IF(F11="","не выбран статус",IF(I11+J11&gt;E11+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F11&lt;&gt;"подписан обеими сторонами",I11&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F11="подписан обеими сторонами",I11+J11=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F11&lt;&gt;"подписан обеими сторонами",G11=""),"Акт не подписан: укажите дату передачи.",IF(AND(F11&lt;&gt;"подписан обеими сторонами",H11=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B11:J11)=0,"",IF(OR(LEN(B11)=0,LEN(C11)=0,LEN(E11)=0,LEN(F11)=0,LEN(I11)=0,LEN(J11)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F11)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E11)),NOT(ISNUMBER(I11)),NOT(ISNUMBER(J11))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E11&lt;0,I11&lt;0,J11&lt;0),"ОШИБКА: отрицательная сумма",IF(I11+J11&gt;E11+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F11&lt;&gt;"подписан обеими сторонами",I11&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F11&lt;&gt;"подписан обеими сторонами",OR(LEN(G11)=0,LEN(H11)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F11&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G11)),G11&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="12" ht="45" customHeight="1">
@@ -1313,11 +1349,12 @@
       <c r="I12" s="17" t="n"/>
       <c r="J12" s="17" t="n"/>
       <c r="K12" s="19">
-        <f>IF(E12="","",ROUND(E12-I12-J12,2))</f>
+        <f>IF(L12="строка заполнена",ROUND(E12-I12-J12,2),"")</f>
         <v/>
       </c>
       <c r="L12" s="15">
-        <f>IF(E12="","",IF(F12="","не выбран статус",IF(I12+J12&gt;E12+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F12&lt;&gt;"подписан обеими сторонами",I12&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F12="подписан обеими сторонами",I12+J12=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F12&lt;&gt;"подписан обеими сторонами",G12=""),"Акт не подписан: укажите дату передачи.",IF(AND(F12&lt;&gt;"подписан обеими сторонами",H12=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B12:J12)=0,"",IF(OR(LEN(B12)=0,LEN(C12)=0,LEN(E12)=0,LEN(F12)=0,LEN(I12)=0,LEN(J12)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F12)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E12)),NOT(ISNUMBER(I12)),NOT(ISNUMBER(J12))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E12&lt;0,I12&lt;0,J12&lt;0),"ОШИБКА: отрицательная сумма",IF(I12+J12&gt;E12+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F12&lt;&gt;"подписан обеими сторонами",I12&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F12&lt;&gt;"подписан обеими сторонами",OR(LEN(G12)=0,LEN(H12)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F12&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G12)),G12&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="13" ht="45" customHeight="1">
@@ -1335,11 +1372,12 @@
       <c r="I13" s="17" t="n"/>
       <c r="J13" s="17" t="n"/>
       <c r="K13" s="19">
-        <f>IF(E13="","",ROUND(E13-I13-J13,2))</f>
+        <f>IF(L13="строка заполнена",ROUND(E13-I13-J13,2),"")</f>
         <v/>
       </c>
       <c r="L13" s="15">
-        <f>IF(E13="","",IF(F13="","не выбран статус",IF(I13+J13&gt;E13+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F13&lt;&gt;"подписан обеими сторонами",I13&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F13="подписан обеими сторонами",I13+J13=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F13&lt;&gt;"подписан обеими сторонами",G13=""),"Акт не подписан: укажите дату передачи.",IF(AND(F13&lt;&gt;"подписан обеими сторонами",H13=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B13:J13)=0,"",IF(OR(LEN(B13)=0,LEN(C13)=0,LEN(E13)=0,LEN(F13)=0,LEN(I13)=0,LEN(J13)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F13)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E13)),NOT(ISNUMBER(I13)),NOT(ISNUMBER(J13))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E13&lt;0,I13&lt;0,J13&lt;0),"ОШИБКА: отрицательная сумма",IF(I13+J13&gt;E13+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F13&lt;&gt;"подписан обеими сторонами",I13&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F13&lt;&gt;"подписан обеими сторонами",OR(LEN(G13)=0,LEN(H13)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F13&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G13)),G13&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="14" ht="45" customHeight="1">
@@ -1357,11 +1395,12 @@
       <c r="I14" s="17" t="n"/>
       <c r="J14" s="17" t="n"/>
       <c r="K14" s="19">
-        <f>IF(E14="","",ROUND(E14-I14-J14,2))</f>
+        <f>IF(L14="строка заполнена",ROUND(E14-I14-J14,2),"")</f>
         <v/>
       </c>
       <c r="L14" s="15">
-        <f>IF(E14="","",IF(F14="","не выбран статус",IF(I14+J14&gt;E14+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F14&lt;&gt;"подписан обеими сторонами",I14&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F14="подписан обеими сторонами",I14+J14=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F14&lt;&gt;"подписан обеими сторонами",G14=""),"Акт не подписан: укажите дату передачи.",IF(AND(F14&lt;&gt;"подписан обеими сторонами",H14=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B14:J14)=0,"",IF(OR(LEN(B14)=0,LEN(C14)=0,LEN(E14)=0,LEN(F14)=0,LEN(I14)=0,LEN(J14)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F14)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E14)),NOT(ISNUMBER(I14)),NOT(ISNUMBER(J14))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E14&lt;0,I14&lt;0,J14&lt;0),"ОШИБКА: отрицательная сумма",IF(I14+J14&gt;E14+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F14&lt;&gt;"подписан обеими сторонами",I14&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F14&lt;&gt;"подписан обеими сторонами",OR(LEN(G14)=0,LEN(H14)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F14&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G14)),G14&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="15" ht="45" customHeight="1">
@@ -1379,11 +1418,12 @@
       <c r="I15" s="17" t="n"/>
       <c r="J15" s="17" t="n"/>
       <c r="K15" s="19">
-        <f>IF(E15="","",ROUND(E15-I15-J15,2))</f>
+        <f>IF(L15="строка заполнена",ROUND(E15-I15-J15,2),"")</f>
         <v/>
       </c>
       <c r="L15" s="15">
-        <f>IF(E15="","",IF(F15="","не выбран статус",IF(I15+J15&gt;E15+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F15&lt;&gt;"подписан обеими сторонами",I15&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F15="подписан обеими сторонами",I15+J15=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F15&lt;&gt;"подписан обеими сторонами",G15=""),"Акт не подписан: укажите дату передачи.",IF(AND(F15&lt;&gt;"подписан обеими сторонами",H15=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B15:J15)=0,"",IF(OR(LEN(B15)=0,LEN(C15)=0,LEN(E15)=0,LEN(F15)=0,LEN(I15)=0,LEN(J15)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F15)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E15)),NOT(ISNUMBER(I15)),NOT(ISNUMBER(J15))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E15&lt;0,I15&lt;0,J15&lt;0),"ОШИБКА: отрицательная сумма",IF(I15+J15&gt;E15+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F15&lt;&gt;"подписан обеими сторонами",I15&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F15&lt;&gt;"подписан обеими сторонами",OR(LEN(G15)=0,LEN(H15)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F15&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G15)),G15&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="16" ht="45" customHeight="1">
@@ -1401,11 +1441,12 @@
       <c r="I16" s="17" t="n"/>
       <c r="J16" s="17" t="n"/>
       <c r="K16" s="19">
-        <f>IF(E16="","",ROUND(E16-I16-J16,2))</f>
+        <f>IF(L16="строка заполнена",ROUND(E16-I16-J16,2),"")</f>
         <v/>
       </c>
       <c r="L16" s="15">
-        <f>IF(E16="","",IF(F16="","не выбран статус",IF(I16+J16&gt;E16+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F16&lt;&gt;"подписан обеими сторонами",I16&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F16="подписан обеими сторонами",I16+J16=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F16&lt;&gt;"подписан обеими сторонами",G16=""),"Акт не подписан: укажите дату передачи.",IF(AND(F16&lt;&gt;"подписан обеими сторонами",H16=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B16:J16)=0,"",IF(OR(LEN(B16)=0,LEN(C16)=0,LEN(E16)=0,LEN(F16)=0,LEN(I16)=0,LEN(J16)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F16)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E16)),NOT(ISNUMBER(I16)),NOT(ISNUMBER(J16))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E16&lt;0,I16&lt;0,J16&lt;0),"ОШИБКА: отрицательная сумма",IF(I16+J16&gt;E16+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F16&lt;&gt;"подписан обеими сторонами",I16&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F16&lt;&gt;"подписан обеими сторонами",OR(LEN(G16)=0,LEN(H16)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F16&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G16)),G16&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="17" ht="45" customHeight="1">
@@ -1423,11 +1464,12 @@
       <c r="I17" s="17" t="n"/>
       <c r="J17" s="17" t="n"/>
       <c r="K17" s="19">
-        <f>IF(E17="","",ROUND(E17-I17-J17,2))</f>
+        <f>IF(L17="строка заполнена",ROUND(E17-I17-J17,2),"")</f>
         <v/>
       </c>
       <c r="L17" s="15">
-        <f>IF(E17="","",IF(F17="","не выбран статус",IF(I17+J17&gt;E17+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F17&lt;&gt;"подписан обеими сторонами",I17&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F17="подписан обеими сторонами",I17+J17=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F17&lt;&gt;"подписан обеими сторонами",G17=""),"Акт не подписан: укажите дату передачи.",IF(AND(F17&lt;&gt;"подписан обеими сторонами",H17=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B17:J17)=0,"",IF(OR(LEN(B17)=0,LEN(C17)=0,LEN(E17)=0,LEN(F17)=0,LEN(I17)=0,LEN(J17)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F17)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E17)),NOT(ISNUMBER(I17)),NOT(ISNUMBER(J17))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E17&lt;0,I17&lt;0,J17&lt;0),"ОШИБКА: отрицательная сумма",IF(I17+J17&gt;E17+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F17&lt;&gt;"подписан обеими сторонами",I17&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F17&lt;&gt;"подписан обеими сторонами",OR(LEN(G17)=0,LEN(H17)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F17&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G17)),G17&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="18" ht="45" customHeight="1">
@@ -1445,11 +1487,12 @@
       <c r="I18" s="17" t="n"/>
       <c r="J18" s="17" t="n"/>
       <c r="K18" s="19">
-        <f>IF(E18="","",ROUND(E18-I18-J18,2))</f>
+        <f>IF(L18="строка заполнена",ROUND(E18-I18-J18,2),"")</f>
         <v/>
       </c>
       <c r="L18" s="15">
-        <f>IF(E18="","",IF(F18="","не выбран статус",IF(I18+J18&gt;E18+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F18&lt;&gt;"подписан обеими сторонами",I18&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F18="подписан обеими сторонами",I18+J18=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F18&lt;&gt;"подписан обеими сторонами",G18=""),"Акт не подписан: укажите дату передачи.",IF(AND(F18&lt;&gt;"подписан обеими сторонами",H18=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B18:J18)=0,"",IF(OR(LEN(B18)=0,LEN(C18)=0,LEN(E18)=0,LEN(F18)=0,LEN(I18)=0,LEN(J18)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F18)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E18)),NOT(ISNUMBER(I18)),NOT(ISNUMBER(J18))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E18&lt;0,I18&lt;0,J18&lt;0),"ОШИБКА: отрицательная сумма",IF(I18+J18&gt;E18+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F18&lt;&gt;"подписан обеими сторонами",I18&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F18&lt;&gt;"подписан обеими сторонами",OR(LEN(G18)=0,LEN(H18)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F18&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G18)),G18&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="19" ht="45" customHeight="1">
@@ -1467,11 +1510,12 @@
       <c r="I19" s="17" t="n"/>
       <c r="J19" s="17" t="n"/>
       <c r="K19" s="19">
-        <f>IF(E19="","",ROUND(E19-I19-J19,2))</f>
+        <f>IF(L19="строка заполнена",ROUND(E19-I19-J19,2),"")</f>
         <v/>
       </c>
       <c r="L19" s="15">
-        <f>IF(E19="","",IF(F19="","не выбран статус",IF(I19+J19&gt;E19+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F19&lt;&gt;"подписан обеими сторонами",I19&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F19="подписан обеими сторонами",I19+J19=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F19&lt;&gt;"подписан обеими сторонами",G19=""),"Акт не подписан: укажите дату передачи.",IF(AND(F19&lt;&gt;"подписан обеими сторонами",H19=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B19:J19)=0,"",IF(OR(LEN(B19)=0,LEN(C19)=0,LEN(E19)=0,LEN(F19)=0,LEN(I19)=0,LEN(J19)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F19)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E19)),NOT(ISNUMBER(I19)),NOT(ISNUMBER(J19))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E19&lt;0,I19&lt;0,J19&lt;0),"ОШИБКА: отрицательная сумма",IF(I19+J19&gt;E19+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F19&lt;&gt;"подписан обеими сторонами",I19&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F19&lt;&gt;"подписан обеими сторонами",OR(LEN(G19)=0,LEN(H19)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F19&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G19)),G19&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="20" ht="45" customHeight="1">
@@ -1489,11 +1533,12 @@
       <c r="I20" s="17" t="n"/>
       <c r="J20" s="17" t="n"/>
       <c r="K20" s="19">
-        <f>IF(E20="","",ROUND(E20-I20-J20,2))</f>
+        <f>IF(L20="строка заполнена",ROUND(E20-I20-J20,2),"")</f>
         <v/>
       </c>
       <c r="L20" s="15">
-        <f>IF(E20="","",IF(F20="","не выбран статус",IF(I20+J20&gt;E20+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F20&lt;&gt;"подписан обеими сторонами",I20&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F20="подписан обеими сторонами",I20+J20=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F20&lt;&gt;"подписан обеими сторонами",G20=""),"Акт не подписан: укажите дату передачи.",IF(AND(F20&lt;&gt;"подписан обеими сторонами",H20=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B20:J20)=0,"",IF(OR(LEN(B20)=0,LEN(C20)=0,LEN(E20)=0,LEN(F20)=0,LEN(I20)=0,LEN(J20)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F20)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E20)),NOT(ISNUMBER(I20)),NOT(ISNUMBER(J20))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E20&lt;0,I20&lt;0,J20&lt;0),"ОШИБКА: отрицательная сумма",IF(I20+J20&gt;E20+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F20&lt;&gt;"подписан обеими сторонами",I20&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F20&lt;&gt;"подписан обеими сторонами",OR(LEN(G20)=0,LEN(H20)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F20&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G20)),G20&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="21" ht="45" customHeight="1">
@@ -1511,11 +1556,12 @@
       <c r="I21" s="17" t="n"/>
       <c r="J21" s="17" t="n"/>
       <c r="K21" s="19">
-        <f>IF(E21="","",ROUND(E21-I21-J21,2))</f>
+        <f>IF(L21="строка заполнена",ROUND(E21-I21-J21,2),"")</f>
         <v/>
       </c>
       <c r="L21" s="15">
-        <f>IF(E21="","",IF(F21="","не выбран статус",IF(I21+J21&gt;E21+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F21&lt;&gt;"подписан обеими сторонами",I21&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F21="подписан обеими сторонами",I21+J21=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F21&lt;&gt;"подписан обеими сторонами",G21=""),"Акт не подписан: укажите дату передачи.",IF(AND(F21&lt;&gt;"подписан обеими сторонами",H21=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B21:J21)=0,"",IF(OR(LEN(B21)=0,LEN(C21)=0,LEN(E21)=0,LEN(F21)=0,LEN(I21)=0,LEN(J21)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F21)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E21)),NOT(ISNUMBER(I21)),NOT(ISNUMBER(J21))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E21&lt;0,I21&lt;0,J21&lt;0),"ОШИБКА: отрицательная сумма",IF(I21+J21&gt;E21+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F21&lt;&gt;"подписан обеими сторонами",I21&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F21&lt;&gt;"подписан обеими сторонами",OR(LEN(G21)=0,LEN(H21)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F21&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G21)),G21&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="22" ht="45" customHeight="1">
@@ -1533,11 +1579,12 @@
       <c r="I22" s="17" t="n"/>
       <c r="J22" s="17" t="n"/>
       <c r="K22" s="19">
-        <f>IF(E22="","",ROUND(E22-I22-J22,2))</f>
+        <f>IF(L22="строка заполнена",ROUND(E22-I22-J22,2),"")</f>
         <v/>
       </c>
       <c r="L22" s="15">
-        <f>IF(E22="","",IF(F22="","не выбран статус",IF(I22+J22&gt;E22+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F22&lt;&gt;"подписан обеими сторонами",I22&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F22="подписан обеими сторонами",I22+J22=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F22&lt;&gt;"подписан обеими сторонами",G22=""),"Акт не подписан: укажите дату передачи.",IF(AND(F22&lt;&gt;"подписан обеими сторонами",H22=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B22:J22)=0,"",IF(OR(LEN(B22)=0,LEN(C22)=0,LEN(E22)=0,LEN(F22)=0,LEN(I22)=0,LEN(J22)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F22)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E22)),NOT(ISNUMBER(I22)),NOT(ISNUMBER(J22))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E22&lt;0,I22&lt;0,J22&lt;0),"ОШИБКА: отрицательная сумма",IF(I22+J22&gt;E22+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F22&lt;&gt;"подписан обеими сторонами",I22&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F22&lt;&gt;"подписан обеими сторонами",OR(LEN(G22)=0,LEN(H22)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F22&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G22)),G22&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="23" ht="45" customHeight="1">
@@ -1555,11 +1602,12 @@
       <c r="I23" s="17" t="n"/>
       <c r="J23" s="17" t="n"/>
       <c r="K23" s="19">
-        <f>IF(E23="","",ROUND(E23-I23-J23,2))</f>
+        <f>IF(L23="строка заполнена",ROUND(E23-I23-J23,2),"")</f>
         <v/>
       </c>
       <c r="L23" s="15">
-        <f>IF(E23="","",IF(F23="","не выбран статус",IF(I23+J23&gt;E23+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F23&lt;&gt;"подписан обеими сторонами",I23&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F23="подписан обеими сторонами",I23+J23=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F23&lt;&gt;"подписан обеими сторонами",G23=""),"Акт не подписан: укажите дату передачи.",IF(AND(F23&lt;&gt;"подписан обеими сторонами",H23=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B23:J23)=0,"",IF(OR(LEN(B23)=0,LEN(C23)=0,LEN(E23)=0,LEN(F23)=0,LEN(I23)=0,LEN(J23)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F23)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E23)),NOT(ISNUMBER(I23)),NOT(ISNUMBER(J23))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E23&lt;0,I23&lt;0,J23&lt;0),"ОШИБКА: отрицательная сумма",IF(I23+J23&gt;E23+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F23&lt;&gt;"подписан обеими сторонами",I23&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F23&lt;&gt;"подписан обеими сторонами",OR(LEN(G23)=0,LEN(H23)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F23&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G23)),G23&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="24" ht="45" customHeight="1">
@@ -1577,11 +1625,12 @@
       <c r="I24" s="17" t="n"/>
       <c r="J24" s="17" t="n"/>
       <c r="K24" s="19">
-        <f>IF(E24="","",ROUND(E24-I24-J24,2))</f>
+        <f>IF(L24="строка заполнена",ROUND(E24-I24-J24,2),"")</f>
         <v/>
       </c>
       <c r="L24" s="15">
-        <f>IF(E24="","",IF(F24="","не выбран статус",IF(I24+J24&gt;E24+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F24&lt;&gt;"подписан обеими сторонами",I24&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F24="подписан обеими сторонами",I24+J24=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F24&lt;&gt;"подписан обеими сторонами",G24=""),"Акт не подписан: укажите дату передачи.",IF(AND(F24&lt;&gt;"подписан обеими сторонами",H24=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B24:J24)=0,"",IF(OR(LEN(B24)=0,LEN(C24)=0,LEN(E24)=0,LEN(F24)=0,LEN(I24)=0,LEN(J24)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F24)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E24)),NOT(ISNUMBER(I24)),NOT(ISNUMBER(J24))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E24&lt;0,I24&lt;0,J24&lt;0),"ОШИБКА: отрицательная сумма",IF(I24+J24&gt;E24+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F24&lt;&gt;"подписан обеими сторонами",I24&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F24&lt;&gt;"подписан обеими сторонами",OR(LEN(G24)=0,LEN(H24)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F24&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G24)),G24&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="25" ht="45" customHeight="1">
@@ -1599,11 +1648,12 @@
       <c r="I25" s="17" t="n"/>
       <c r="J25" s="17" t="n"/>
       <c r="K25" s="19">
-        <f>IF(E25="","",ROUND(E25-I25-J25,2))</f>
+        <f>IF(L25="строка заполнена",ROUND(E25-I25-J25,2),"")</f>
         <v/>
       </c>
       <c r="L25" s="15">
-        <f>IF(E25="","",IF(F25="","не выбран статус",IF(I25+J25&gt;E25+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F25&lt;&gt;"подписан обеими сторонами",I25&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F25="подписан обеими сторонами",I25+J25=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F25&lt;&gt;"подписан обеими сторонами",G25=""),"Акт не подписан: укажите дату передачи.",IF(AND(F25&lt;&gt;"подписан обеими сторонами",H25=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B25:J25)=0,"",IF(OR(LEN(B25)=0,LEN(C25)=0,LEN(E25)=0,LEN(F25)=0,LEN(I25)=0,LEN(J25)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F25)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E25)),NOT(ISNUMBER(I25)),NOT(ISNUMBER(J25))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E25&lt;0,I25&lt;0,J25&lt;0),"ОШИБКА: отрицательная сумма",IF(I25+J25&gt;E25+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F25&lt;&gt;"подписан обеими сторонами",I25&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F25&lt;&gt;"подписан обеими сторонами",OR(LEN(G25)=0,LEN(H25)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F25&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G25)),G25&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="26" ht="45" customHeight="1">
@@ -1621,11 +1671,12 @@
       <c r="I26" s="17" t="n"/>
       <c r="J26" s="17" t="n"/>
       <c r="K26" s="19">
-        <f>IF(E26="","",ROUND(E26-I26-J26,2))</f>
+        <f>IF(L26="строка заполнена",ROUND(E26-I26-J26,2),"")</f>
         <v/>
       </c>
       <c r="L26" s="15">
-        <f>IF(E26="","",IF(F26="","не выбран статус",IF(I26+J26&gt;E26+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F26&lt;&gt;"подписан обеими сторонами",I26&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F26="подписан обеими сторонами",I26+J26=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F26&lt;&gt;"подписан обеими сторонами",G26=""),"Акт не подписан: укажите дату передачи.",IF(AND(F26&lt;&gt;"подписан обеими сторонами",H26=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B26:J26)=0,"",IF(OR(LEN(B26)=0,LEN(C26)=0,LEN(E26)=0,LEN(F26)=0,LEN(I26)=0,LEN(J26)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F26)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E26)),NOT(ISNUMBER(I26)),NOT(ISNUMBER(J26))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E26&lt;0,I26&lt;0,J26&lt;0),"ОШИБКА: отрицательная сумма",IF(I26+J26&gt;E26+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F26&lt;&gt;"подписан обеими сторонами",I26&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F26&lt;&gt;"подписан обеими сторонами",OR(LEN(G26)=0,LEN(H26)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F26&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G26)),G26&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="27" ht="45" customHeight="1">
@@ -1643,11 +1694,12 @@
       <c r="I27" s="17" t="n"/>
       <c r="J27" s="17" t="n"/>
       <c r="K27" s="19">
-        <f>IF(E27="","",ROUND(E27-I27-J27,2))</f>
+        <f>IF(L27="строка заполнена",ROUND(E27-I27-J27,2),"")</f>
         <v/>
       </c>
       <c r="L27" s="15">
-        <f>IF(E27="","",IF(F27="","не выбран статус",IF(I27+J27&gt;E27+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F27&lt;&gt;"подписан обеими сторонами",I27&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F27="подписан обеими сторонами",I27+J27=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F27&lt;&gt;"подписан обеими сторонами",G27=""),"Акт не подписан: укажите дату передачи.",IF(AND(F27&lt;&gt;"подписан обеими сторонами",H27=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B27:J27)=0,"",IF(OR(LEN(B27)=0,LEN(C27)=0,LEN(E27)=0,LEN(F27)=0,LEN(I27)=0,LEN(J27)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F27)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E27)),NOT(ISNUMBER(I27)),NOT(ISNUMBER(J27))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E27&lt;0,I27&lt;0,J27&lt;0),"ОШИБКА: отрицательная сумма",IF(I27+J27&gt;E27+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F27&lt;&gt;"подписан обеими сторонами",I27&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F27&lt;&gt;"подписан обеими сторонами",OR(LEN(G27)=0,LEN(H27)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F27&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G27)),G27&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="28" ht="45" customHeight="1">
@@ -1665,11 +1717,12 @@
       <c r="I28" s="17" t="n"/>
       <c r="J28" s="17" t="n"/>
       <c r="K28" s="19">
-        <f>IF(E28="","",ROUND(E28-I28-J28,2))</f>
+        <f>IF(L28="строка заполнена",ROUND(E28-I28-J28,2),"")</f>
         <v/>
       </c>
       <c r="L28" s="15">
-        <f>IF(E28="","",IF(F28="","не выбран статус",IF(I28+J28&gt;E28+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F28&lt;&gt;"подписан обеими сторонами",I28&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F28="подписан обеими сторонами",I28+J28=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F28&lt;&gt;"подписан обеими сторонами",G28=""),"Акт не подписан: укажите дату передачи.",IF(AND(F28&lt;&gt;"подписан обеими сторонами",H28=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B28:J28)=0,"",IF(OR(LEN(B28)=0,LEN(C28)=0,LEN(E28)=0,LEN(F28)=0,LEN(I28)=0,LEN(J28)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F28)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E28)),NOT(ISNUMBER(I28)),NOT(ISNUMBER(J28))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E28&lt;0,I28&lt;0,J28&lt;0),"ОШИБКА: отрицательная сумма",IF(I28+J28&gt;E28+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F28&lt;&gt;"подписан обеими сторонами",I28&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F28&lt;&gt;"подписан обеими сторонами",OR(LEN(G28)=0,LEN(H28)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F28&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G28)),G28&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="29" ht="45" customHeight="1">
@@ -1687,11 +1740,12 @@
       <c r="I29" s="17" t="n"/>
       <c r="J29" s="17" t="n"/>
       <c r="K29" s="19">
-        <f>IF(E29="","",ROUND(E29-I29-J29,2))</f>
+        <f>IF(L29="строка заполнена",ROUND(E29-I29-J29,2),"")</f>
         <v/>
       </c>
       <c r="L29" s="15">
-        <f>IF(E29="","",IF(F29="","не выбран статус",IF(I29+J29&gt;E29+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F29&lt;&gt;"подписан обеими сторонами",I29&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F29="подписан обеими сторонами",I29+J29=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F29&lt;&gt;"подписан обеими сторонами",G29=""),"Акт не подписан: укажите дату передачи.",IF(AND(F29&lt;&gt;"подписан обеими сторонами",H29=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B29:J29)=0,"",IF(OR(LEN(B29)=0,LEN(C29)=0,LEN(E29)=0,LEN(F29)=0,LEN(I29)=0,LEN(J29)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F29)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E29)),NOT(ISNUMBER(I29)),NOT(ISNUMBER(J29))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E29&lt;0,I29&lt;0,J29&lt;0),"ОШИБКА: отрицательная сумма",IF(I29+J29&gt;E29+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F29&lt;&gt;"подписан обеими сторонами",I29&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F29&lt;&gt;"подписан обеими сторонами",OR(LEN(G29)=0,LEN(H29)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F29&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G29)),G29&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="30" ht="45" customHeight="1">
@@ -1709,11 +1763,12 @@
       <c r="I30" s="17" t="n"/>
       <c r="J30" s="17" t="n"/>
       <c r="K30" s="19">
-        <f>IF(E30="","",ROUND(E30-I30-J30,2))</f>
+        <f>IF(L30="строка заполнена",ROUND(E30-I30-J30,2),"")</f>
         <v/>
       </c>
       <c r="L30" s="15">
-        <f>IF(E30="","",IF(F30="","не выбран статус",IF(I30+J30&gt;E30+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F30&lt;&gt;"подписан обеими сторонами",I30&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F30="подписан обеими сторонами",I30+J30=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F30&lt;&gt;"подписан обеими сторонами",G30=""),"Акт не подписан: укажите дату передачи.",IF(AND(F30&lt;&gt;"подписан обеими сторонами",H30=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B30:J30)=0,"",IF(OR(LEN(B30)=0,LEN(C30)=0,LEN(E30)=0,LEN(F30)=0,LEN(I30)=0,LEN(J30)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F30)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E30)),NOT(ISNUMBER(I30)),NOT(ISNUMBER(J30))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E30&lt;0,I30&lt;0,J30&lt;0),"ОШИБКА: отрицательная сумма",IF(I30+J30&gt;E30+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F30&lt;&gt;"подписан обеими сторонами",I30&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F30&lt;&gt;"подписан обеими сторонами",OR(LEN(G30)=0,LEN(H30)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F30&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G30)),G30&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="31" ht="45" customHeight="1">
@@ -1731,11 +1786,12 @@
       <c r="I31" s="17" t="n"/>
       <c r="J31" s="17" t="n"/>
       <c r="K31" s="19">
-        <f>IF(E31="","",ROUND(E31-I31-J31,2))</f>
+        <f>IF(L31="строка заполнена",ROUND(E31-I31-J31,2),"")</f>
         <v/>
       </c>
       <c r="L31" s="15">
-        <f>IF(E31="","",IF(F31="","не выбран статус",IF(I31+J31&gt;E31+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F31&lt;&gt;"подписан обеими сторонами",I31&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F31="подписан обеими сторонами",I31+J31=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F31&lt;&gt;"подписан обеими сторонами",G31=""),"Акт не подписан: укажите дату передачи.",IF(AND(F31&lt;&gt;"подписан обеими сторонами",H31=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B31:J31)=0,"",IF(OR(LEN(B31)=0,LEN(C31)=0,LEN(E31)=0,LEN(F31)=0,LEN(I31)=0,LEN(J31)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F31)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E31)),NOT(ISNUMBER(I31)),NOT(ISNUMBER(J31))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E31&lt;0,I31&lt;0,J31&lt;0),"ОШИБКА: отрицательная сумма",IF(I31+J31&gt;E31+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F31&lt;&gt;"подписан обеими сторонами",I31&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F31&lt;&gt;"подписан обеими сторонами",OR(LEN(G31)=0,LEN(H31)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F31&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G31)),G31&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="32" ht="45" customHeight="1">
@@ -1753,11 +1809,12 @@
       <c r="I32" s="17" t="n"/>
       <c r="J32" s="17" t="n"/>
       <c r="K32" s="19">
-        <f>IF(E32="","",ROUND(E32-I32-J32,2))</f>
+        <f>IF(L32="строка заполнена",ROUND(E32-I32-J32,2),"")</f>
         <v/>
       </c>
       <c r="L32" s="15">
-        <f>IF(E32="","",IF(F32="","не выбран статус",IF(I32+J32&gt;E32+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F32&lt;&gt;"подписан обеими сторонами",I32&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F32="подписан обеими сторонами",I32+J32=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F32&lt;&gt;"подписан обеими сторонами",G32=""),"Акт не подписан: укажите дату передачи.",IF(AND(F32&lt;&gt;"подписан обеими сторонами",H32=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B32:J32)=0,"",IF(OR(LEN(B32)=0,LEN(C32)=0,LEN(E32)=0,LEN(F32)=0,LEN(I32)=0,LEN(J32)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F32)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E32)),NOT(ISNUMBER(I32)),NOT(ISNUMBER(J32))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E32&lt;0,I32&lt;0,J32&lt;0),"ОШИБКА: отрицательная сумма",IF(I32+J32&gt;E32+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F32&lt;&gt;"подписан обеими сторонами",I32&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F32&lt;&gt;"подписан обеими сторонами",OR(LEN(G32)=0,LEN(H32)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F32&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G32)),G32&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="33" ht="45" customHeight="1">
@@ -1775,11 +1832,12 @@
       <c r="I33" s="17" t="n"/>
       <c r="J33" s="17" t="n"/>
       <c r="K33" s="19">
-        <f>IF(E33="","",ROUND(E33-I33-J33,2))</f>
+        <f>IF(L33="строка заполнена",ROUND(E33-I33-J33,2),"")</f>
         <v/>
       </c>
       <c r="L33" s="15">
-        <f>IF(E33="","",IF(F33="","не выбран статус",IF(I33+J33&gt;E33+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F33&lt;&gt;"подписан обеими сторонами",I33&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F33="подписан обеими сторонами",I33+J33=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F33&lt;&gt;"подписан обеими сторонами",G33=""),"Акт не подписан: укажите дату передачи.",IF(AND(F33&lt;&gt;"подписан обеими сторонами",H33=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B33:J33)=0,"",IF(OR(LEN(B33)=0,LEN(C33)=0,LEN(E33)=0,LEN(F33)=0,LEN(I33)=0,LEN(J33)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F33)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E33)),NOT(ISNUMBER(I33)),NOT(ISNUMBER(J33))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E33&lt;0,I33&lt;0,J33&lt;0),"ОШИБКА: отрицательная сумма",IF(I33+J33&gt;E33+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F33&lt;&gt;"подписан обеими сторонами",I33&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F33&lt;&gt;"подписан обеими сторонами",OR(LEN(G33)=0,LEN(H33)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F33&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G33)),G33&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="34" ht="45" customHeight="1">
@@ -1797,11 +1855,12 @@
       <c r="I34" s="17" t="n"/>
       <c r="J34" s="17" t="n"/>
       <c r="K34" s="19">
-        <f>IF(E34="","",ROUND(E34-I34-J34,2))</f>
+        <f>IF(L34="строка заполнена",ROUND(E34-I34-J34,2),"")</f>
         <v/>
       </c>
       <c r="L34" s="15">
-        <f>IF(E34="","",IF(F34="","не выбран статус",IF(I34+J34&gt;E34+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F34&lt;&gt;"подписан обеими сторонами",I34&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F34="подписан обеими сторонами",I34+J34=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F34&lt;&gt;"подписан обеими сторонами",G34=""),"Акт не подписан: укажите дату передачи.",IF(AND(F34&lt;&gt;"подписан обеими сторонами",H34=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B34:J34)=0,"",IF(OR(LEN(B34)=0,LEN(C34)=0,LEN(E34)=0,LEN(F34)=0,LEN(I34)=0,LEN(J34)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F34)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E34)),NOT(ISNUMBER(I34)),NOT(ISNUMBER(J34))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E34&lt;0,I34&lt;0,J34&lt;0),"ОШИБКА: отрицательная сумма",IF(I34+J34&gt;E34+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F34&lt;&gt;"подписан обеими сторонами",I34&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F34&lt;&gt;"подписан обеими сторонами",OR(LEN(G34)=0,LEN(H34)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F34&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G34)),G34&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="35" ht="45" customHeight="1">
@@ -1819,11 +1878,12 @@
       <c r="I35" s="17" t="n"/>
       <c r="J35" s="17" t="n"/>
       <c r="K35" s="19">
-        <f>IF(E35="","",ROUND(E35-I35-J35,2))</f>
+        <f>IF(L35="строка заполнена",ROUND(E35-I35-J35,2),"")</f>
         <v/>
       </c>
       <c r="L35" s="15">
-        <f>IF(E35="","",IF(F35="","не выбран статус",IF(I35+J35&gt;E35+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F35&lt;&gt;"подписан обеими сторонами",I35&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F35="подписан обеими сторонами",I35+J35=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F35&lt;&gt;"подписан обеими сторонами",G35=""),"Акт не подписан: укажите дату передачи.",IF(AND(F35&lt;&gt;"подписан обеими сторонами",H35=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B35:J35)=0,"",IF(OR(LEN(B35)=0,LEN(C35)=0,LEN(E35)=0,LEN(F35)=0,LEN(I35)=0,LEN(J35)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F35)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E35)),NOT(ISNUMBER(I35)),NOT(ISNUMBER(J35))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E35&lt;0,I35&lt;0,J35&lt;0),"ОШИБКА: отрицательная сумма",IF(I35+J35&gt;E35+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F35&lt;&gt;"подписан обеими сторонами",I35&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F35&lt;&gt;"подписан обеими сторонами",OR(LEN(G35)=0,LEN(H35)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F35&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G35)),G35&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="36" ht="45" customHeight="1">
@@ -1841,11 +1901,12 @@
       <c r="I36" s="17" t="n"/>
       <c r="J36" s="17" t="n"/>
       <c r="K36" s="19">
-        <f>IF(E36="","",ROUND(E36-I36-J36,2))</f>
+        <f>IF(L36="строка заполнена",ROUND(E36-I36-J36,2),"")</f>
         <v/>
       </c>
       <c r="L36" s="15">
-        <f>IF(E36="","",IF(F36="","не выбран статус",IF(I36+J36&gt;E36+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F36&lt;&gt;"подписан обеими сторонами",I36&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F36="подписан обеими сторонами",I36+J36=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F36&lt;&gt;"подписан обеими сторонами",G36=""),"Акт не подписан: укажите дату передачи.",IF(AND(F36&lt;&gt;"подписан обеими сторонами",H36=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B36:J36)=0,"",IF(OR(LEN(B36)=0,LEN(C36)=0,LEN(E36)=0,LEN(F36)=0,LEN(I36)=0,LEN(J36)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F36)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E36)),NOT(ISNUMBER(I36)),NOT(ISNUMBER(J36))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E36&lt;0,I36&lt;0,J36&lt;0),"ОШИБКА: отрицательная сумма",IF(I36+J36&gt;E36+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F36&lt;&gt;"подписан обеими сторонами",I36&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F36&lt;&gt;"подписан обеими сторонами",OR(LEN(G36)=0,LEN(H36)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F36&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G36)),G36&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="37" ht="45" customHeight="1">
@@ -1863,11 +1924,12 @@
       <c r="I37" s="17" t="n"/>
       <c r="J37" s="17" t="n"/>
       <c r="K37" s="19">
-        <f>IF(E37="","",ROUND(E37-I37-J37,2))</f>
+        <f>IF(L37="строка заполнена",ROUND(E37-I37-J37,2),"")</f>
         <v/>
       </c>
       <c r="L37" s="15">
-        <f>IF(E37="","",IF(F37="","не выбран статус",IF(I37+J37&gt;E37+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F37&lt;&gt;"подписан обеими сторонами",I37&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F37="подписан обеими сторонами",I37+J37=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F37&lt;&gt;"подписан обеими сторонами",G37=""),"Акт не подписан: укажите дату передачи.",IF(AND(F37&lt;&gt;"подписан обеими сторонами",H37=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B37:J37)=0,"",IF(OR(LEN(B37)=0,LEN(C37)=0,LEN(E37)=0,LEN(F37)=0,LEN(I37)=0,LEN(J37)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F37)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E37)),NOT(ISNUMBER(I37)),NOT(ISNUMBER(J37))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E37&lt;0,I37&lt;0,J37&lt;0),"ОШИБКА: отрицательная сумма",IF(I37+J37&gt;E37+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F37&lt;&gt;"подписан обеими сторонами",I37&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F37&lt;&gt;"подписан обеими сторонами",OR(LEN(G37)=0,LEN(H37)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F37&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G37)),G37&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="38" ht="45" customHeight="1">
@@ -1885,11 +1947,12 @@
       <c r="I38" s="17" t="n"/>
       <c r="J38" s="17" t="n"/>
       <c r="K38" s="19">
-        <f>IF(E38="","",ROUND(E38-I38-J38,2))</f>
+        <f>IF(L38="строка заполнена",ROUND(E38-I38-J38,2),"")</f>
         <v/>
       </c>
       <c r="L38" s="15">
-        <f>IF(E38="","",IF(F38="","не выбран статус",IF(I38+J38&gt;E38+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F38&lt;&gt;"подписан обеими сторонами",I38&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F38="подписан обеими сторонами",I38+J38=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F38&lt;&gt;"подписан обеими сторонами",G38=""),"Акт не подписан: укажите дату передачи.",IF(AND(F38&lt;&gt;"подписан обеими сторонами",H38=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B38:J38)=0,"",IF(OR(LEN(B38)=0,LEN(C38)=0,LEN(E38)=0,LEN(F38)=0,LEN(I38)=0,LEN(J38)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F38)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E38)),NOT(ISNUMBER(I38)),NOT(ISNUMBER(J38))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E38&lt;0,I38&lt;0,J38&lt;0),"ОШИБКА: отрицательная сумма",IF(I38+J38&gt;E38+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F38&lt;&gt;"подписан обеими сторонами",I38&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F38&lt;&gt;"подписан обеими сторонами",OR(LEN(G38)=0,LEN(H38)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F38&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G38)),G38&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="39" ht="45" customHeight="1">
@@ -1907,11 +1970,12 @@
       <c r="I39" s="17" t="n"/>
       <c r="J39" s="17" t="n"/>
       <c r="K39" s="19">
-        <f>IF(E39="","",ROUND(E39-I39-J39,2))</f>
+        <f>IF(L39="строка заполнена",ROUND(E39-I39-J39,2),"")</f>
         <v/>
       </c>
       <c r="L39" s="15">
-        <f>IF(E39="","",IF(F39="","не выбран статус",IF(I39+J39&gt;E39+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F39&lt;&gt;"подписан обеими сторонами",I39&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F39="подписан обеими сторонами",I39+J39=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F39&lt;&gt;"подписан обеими сторонами",G39=""),"Акт не подписан: укажите дату передачи.",IF(AND(F39&lt;&gt;"подписан обеими сторонами",H39=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B39:J39)=0,"",IF(OR(LEN(B39)=0,LEN(C39)=0,LEN(E39)=0,LEN(F39)=0,LEN(I39)=0,LEN(J39)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F39)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E39)),NOT(ISNUMBER(I39)),NOT(ISNUMBER(J39))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E39&lt;0,I39&lt;0,J39&lt;0),"ОШИБКА: отрицательная сумма",IF(I39+J39&gt;E39+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F39&lt;&gt;"подписан обеими сторонами",I39&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F39&lt;&gt;"подписан обеими сторонами",OR(LEN(G39)=0,LEN(H39)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F39&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G39)),G39&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="40" ht="45" customHeight="1">
@@ -1929,11 +1993,12 @@
       <c r="I40" s="17" t="n"/>
       <c r="J40" s="17" t="n"/>
       <c r="K40" s="19">
-        <f>IF(E40="","",ROUND(E40-I40-J40,2))</f>
+        <f>IF(L40="строка заполнена",ROUND(E40-I40-J40,2),"")</f>
         <v/>
       </c>
       <c r="L40" s="15">
-        <f>IF(E40="","",IF(F40="","не выбран статус",IF(I40+J40&gt;E40+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F40&lt;&gt;"подписан обеими сторонами",I40&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F40="подписан обеими сторонами",I40+J40=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F40&lt;&gt;"подписан обеими сторонами",G40=""),"Акт не подписан: укажите дату передачи.",IF(AND(F40&lt;&gt;"подписан обеими сторонами",H40=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B40:J40)=0,"",IF(OR(LEN(B40)=0,LEN(C40)=0,LEN(E40)=0,LEN(F40)=0,LEN(I40)=0,LEN(J40)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F40)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E40)),NOT(ISNUMBER(I40)),NOT(ISNUMBER(J40))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E40&lt;0,I40&lt;0,J40&lt;0),"ОШИБКА: отрицательная сумма",IF(I40+J40&gt;E40+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F40&lt;&gt;"подписан обеими сторонами",I40&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F40&lt;&gt;"подписан обеими сторонами",OR(LEN(G40)=0,LEN(H40)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F40&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G40)),G40&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="41" ht="45" customHeight="1">
@@ -1951,11 +2016,12 @@
       <c r="I41" s="17" t="n"/>
       <c r="J41" s="17" t="n"/>
       <c r="K41" s="19">
-        <f>IF(E41="","",ROUND(E41-I41-J41,2))</f>
+        <f>IF(L41="строка заполнена",ROUND(E41-I41-J41,2),"")</f>
         <v/>
       </c>
       <c r="L41" s="15">
-        <f>IF(E41="","",IF(F41="","не выбран статус",IF(I41+J41&gt;E41+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F41&lt;&gt;"подписан обеими сторонами",I41&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F41="подписан обеими сторонами",I41+J41=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F41&lt;&gt;"подписан обеими сторонами",G41=""),"Акт не подписан: укажите дату передачи.",IF(AND(F41&lt;&gt;"подписан обеими сторонами",H41=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B41:J41)=0,"",IF(OR(LEN(B41)=0,LEN(C41)=0,LEN(E41)=0,LEN(F41)=0,LEN(I41)=0,LEN(J41)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F41)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E41)),NOT(ISNUMBER(I41)),NOT(ISNUMBER(J41))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E41&lt;0,I41&lt;0,J41&lt;0),"ОШИБКА: отрицательная сумма",IF(I41+J41&gt;E41+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F41&lt;&gt;"подписан обеими сторонами",I41&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F41&lt;&gt;"подписан обеими сторонами",OR(LEN(G41)=0,LEN(H41)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F41&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G41)),G41&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="42" ht="45" customHeight="1">
@@ -1973,11 +2039,12 @@
       <c r="I42" s="17" t="n"/>
       <c r="J42" s="17" t="n"/>
       <c r="K42" s="19">
-        <f>IF(E42="","",ROUND(E42-I42-J42,2))</f>
+        <f>IF(L42="строка заполнена",ROUND(E42-I42-J42,2),"")</f>
         <v/>
       </c>
       <c r="L42" s="15">
-        <f>IF(E42="","",IF(F42="","не выбран статус",IF(I42+J42&gt;E42+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F42&lt;&gt;"подписан обеими сторонами",I42&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F42="подписан обеими сторонами",I42+J42=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F42&lt;&gt;"подписан обеими сторонами",G42=""),"Акт не подписан: укажите дату передачи.",IF(AND(F42&lt;&gt;"подписан обеими сторонами",H42=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B42:J42)=0,"",IF(OR(LEN(B42)=0,LEN(C42)=0,LEN(E42)=0,LEN(F42)=0,LEN(I42)=0,LEN(J42)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F42)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E42)),NOT(ISNUMBER(I42)),NOT(ISNUMBER(J42))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E42&lt;0,I42&lt;0,J42&lt;0),"ОШИБКА: отрицательная сумма",IF(I42+J42&gt;E42+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F42&lt;&gt;"подписан обеими сторонами",I42&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F42&lt;&gt;"подписан обеими сторонами",OR(LEN(G42)=0,LEN(H42)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F42&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G42)),G42&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="43" ht="45" customHeight="1">
@@ -1995,11 +2062,12 @@
       <c r="I43" s="17" t="n"/>
       <c r="J43" s="17" t="n"/>
       <c r="K43" s="19">
-        <f>IF(E43="","",ROUND(E43-I43-J43,2))</f>
+        <f>IF(L43="строка заполнена",ROUND(E43-I43-J43,2),"")</f>
         <v/>
       </c>
       <c r="L43" s="15">
-        <f>IF(E43="","",IF(F43="","не выбран статус",IF(I43+J43&gt;E43+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F43&lt;&gt;"подписан обеими сторонами",I43&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F43="подписан обеими сторонами",I43+J43=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F43&lt;&gt;"подписан обеими сторонами",G43=""),"Акт не подписан: укажите дату передачи.",IF(AND(F43&lt;&gt;"подписан обеими сторонами",H43=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B43:J43)=0,"",IF(OR(LEN(B43)=0,LEN(C43)=0,LEN(E43)=0,LEN(F43)=0,LEN(I43)=0,LEN(J43)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F43)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E43)),NOT(ISNUMBER(I43)),NOT(ISNUMBER(J43))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E43&lt;0,I43&lt;0,J43&lt;0),"ОШИБКА: отрицательная сумма",IF(I43+J43&gt;E43+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F43&lt;&gt;"подписан обеими сторонами",I43&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F43&lt;&gt;"подписан обеими сторонами",OR(LEN(G43)=0,LEN(H43)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F43&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G43)),G43&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="44" ht="45" customHeight="1">
@@ -2017,11 +2085,12 @@
       <c r="I44" s="17" t="n"/>
       <c r="J44" s="17" t="n"/>
       <c r="K44" s="19">
-        <f>IF(E44="","",ROUND(E44-I44-J44,2))</f>
+        <f>IF(L44="строка заполнена",ROUND(E44-I44-J44,2),"")</f>
         <v/>
       </c>
       <c r="L44" s="15">
-        <f>IF(E44="","",IF(F44="","не выбран статус",IF(I44+J44&gt;E44+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F44&lt;&gt;"подписан обеими сторонами",I44&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F44="подписан обеими сторонами",I44+J44=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F44&lt;&gt;"подписан обеими сторонами",G44=""),"Акт не подписан: укажите дату передачи.",IF(AND(F44&lt;&gt;"подписан обеими сторонами",H44=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B44:J44)=0,"",IF(OR(LEN(B44)=0,LEN(C44)=0,LEN(E44)=0,LEN(F44)=0,LEN(I44)=0,LEN(J44)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F44)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E44)),NOT(ISNUMBER(I44)),NOT(ISNUMBER(J44))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E44&lt;0,I44&lt;0,J44&lt;0),"ОШИБКА: отрицательная сумма",IF(I44+J44&gt;E44+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F44&lt;&gt;"подписан обеими сторонами",I44&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F44&lt;&gt;"подписан обеими сторонами",OR(LEN(G44)=0,LEN(H44)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F44&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G44)),G44&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="45" ht="45" customHeight="1">
@@ -2039,11 +2108,12 @@
       <c r="I45" s="17" t="n"/>
       <c r="J45" s="17" t="n"/>
       <c r="K45" s="19">
-        <f>IF(E45="","",ROUND(E45-I45-J45,2))</f>
+        <f>IF(L45="строка заполнена",ROUND(E45-I45-J45,2),"")</f>
         <v/>
       </c>
       <c r="L45" s="15">
-        <f>IF(E45="","",IF(F45="","не выбран статус",IF(I45+J45&gt;E45+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F45&lt;&gt;"подписан обеими сторонами",I45&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F45="подписан обеими сторонами",I45+J45=0),"По подписанному акту не отражены погашение аванса и оплата: проверьте платежи.",IF(AND(F45&lt;&gt;"подписан обеими сторонами",G45=""),"Акт не подписан: укажите дату передачи.",IF(AND(F45&lt;&gt;"подписан обеими сторонами",H45=""),"Акт не подписан: укажите документ, подтверждающий передачу.","строка заполнена")))))))</f>
+        <f>IF(COUNTA(B45:J45)=0,"",IF(OR(LEN(B45)=0,LEN(C45)=0,LEN(E45)=0,LEN(F45)=0,LEN(I45)=0,LEN(J45)=0),"НЕ ЗАПОЛНЕНО: документ, номер, стоимость, статус и оплаты (ноль числом)",IF(COUNTIF($N$2:$N$5,F45)&lt;&gt;1,"ОШИБКА: неизвестный статус акта",IF(OR(NOT(ISNUMBER(E45)),NOT(ISNUMBER(I45)),NOT(ISNUMBER(J45))),"ОШИБКА: стоимость и оплаты должны быть числами",IF(OR(E45&lt;0,I45&lt;0,J45&lt;0),"ОШИБКА: отрицательная сумма",IF(I45+J45&gt;E45+0.01,"ОШИБКА: погашение аванса и оплата превышают стоимость акта.",IF(AND(F45&lt;&gt;"подписан обеими сторонами",I45&gt;0),"ОШИБКА: погашение аванса отнесено к акту, не подписанному обеими сторонами.",IF(AND(F45&lt;&gt;"подписан обеими сторонами",OR(LEN(G45)=0,LEN(H45)=0)),"НЕ ЗАПОЛНЕНО: дата и подтверждение передачи акта",IF(AND(F45&lt;&gt;"подписан обеими сторонами",OR(NOT(ISNUMBER(G45)),G45&lt;=0)),"ОШИБКА: дата передачи должна быть датой Excel","строка заполнена")))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="46">
@@ -2144,18 +2214,18 @@
     <row r="55">
       <c r="A55" s="20" t="inlineStr">
         <is>
-          <t>Строк с ошибкой в колонке «Проверка»</t>
+          <t>Строк с ошибками или незаполненными данными</t>
         </is>
       </c>
       <c r="E55" s="21">
-        <f>COUNTIF(L6:L45,"ОШИБКА*")</f>
+        <f>SUMPRODUCT(--(LEFT(L6:L45,6)="ОШИБКА"))+SUMPRODUCT(--(LEFT(L6:L45,12)="НЕ ЗАПОЛНЕНО"))</f>
         <v/>
       </c>
     </row>
     <row r="57" ht="60" customHeight="1">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>Колонка «Не оплачено» показывает стоимость акта за вычетом погашенного аванса и денежной оплаты. Сверьте каждую строку с актом и платежом.</t>
+          <t>Не оплачено = стоимость − погашение аванса − денежная оплата. Незавершённая строка блокирует итог сальдо; её данные нужно проверить, а не удалять из расчёта.</t>
         </is>
       </c>
     </row>
@@ -2176,8 +2246,8 @@
     <mergeCell ref="A47:D47"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="F6:F45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Выберите статус акта из списка" type="list">
-      <formula1>"подписан обеими сторонами,передан, не подписан,подписан односторонне,получен мотивированный отказ"</formula1>
+    <dataValidation type="list" errorStyle="stop" allowBlank="0" showDropDown="0" showErrorMessage="1" errorTitle="Статус акта" error="Выберите один из четырёх статусов списка." sqref="F6:F45">
+      <formula1>$N$2:$N$5</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2266,7 +2336,8 @@
       <c r="E6" s="16" t="n"/>
       <c r="F6" s="16" t="n"/>
       <c r="G6" s="15">
-        <f>IF(D6="","",IF(B6="","не выбрано основание",IF(E6="","ОШИБКА: сумма без подтверждающего документа",IF(F6="","не указано, подписан ли документ второй стороной",IF(F6="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
+        <f>IF(COUNTA(B6:F6)=0,"",IF(OR(LEN(B6)=0,LEN(C6)=0,LEN(D6)=0,LEN(E6)=0,LEN(F6)=0),"НЕ ЗАПОЛНЕНО: основание, описание, сумма, документ и подпись",IF(NOT(OR(B6="материалы переданы генподрядчику",B6="материалы и оборудование остались на объекте",B6="затраты на мобилизацию и демобилизацию",B6="гарантийное удержание из оплаченных актов",B6="иное")),"ОШИБКА: неизвестное основание встречной суммы",IF(NOT(ISNUMBER(D6)),"ОШИБКА: сумма должна быть числом",IF(D6&lt;0,"ОШИБКА: отрицательная сумма",IF(AND(F6&lt;&gt;"да",F6&lt;&gt;"нет"),"ОШИБКА: подпись — выберите да или нет",IF(F6="нет","ПРОВЕРЬТЕ: самостоятельное основание и доказательства","строка заполнена")))))))</f>
+        <v/>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
@@ -2280,7 +2351,8 @@
       <c r="E7" s="16" t="n"/>
       <c r="F7" s="16" t="n"/>
       <c r="G7" s="15">
-        <f>IF(D7="","",IF(B7="","не выбрано основание",IF(E7="","ОШИБКА: сумма без подтверждающего документа",IF(F7="","не указано, подписан ли документ второй стороной",IF(F7="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
+        <f>IF(COUNTA(B7:F7)=0,"",IF(OR(LEN(B7)=0,LEN(C7)=0,LEN(D7)=0,LEN(E7)=0,LEN(F7)=0),"НЕ ЗАПОЛНЕНО: основание, описание, сумма, документ и подпись",IF(NOT(OR(B7="материалы переданы генподрядчику",B7="материалы и оборудование остались на объекте",B7="затраты на мобилизацию и демобилизацию",B7="гарантийное удержание из оплаченных актов",B7="иное")),"ОШИБКА: неизвестное основание встречной суммы",IF(NOT(ISNUMBER(D7)),"ОШИБКА: сумма должна быть числом",IF(D7&lt;0,"ОШИБКА: отрицательная сумма",IF(AND(F7&lt;&gt;"да",F7&lt;&gt;"нет"),"ОШИБКА: подпись — выберите да или нет",IF(F7="нет","ПРОВЕРЬТЕ: самостоятельное основание и доказательства","строка заполнена")))))))</f>
+        <v/>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1">
@@ -2294,7 +2366,8 @@
       <c r="E8" s="16" t="n"/>
       <c r="F8" s="16" t="n"/>
       <c r="G8" s="15">
-        <f>IF(D8="","",IF(B8="","не выбрано основание",IF(E8="","ОШИБКА: сумма без подтверждающего документа",IF(F8="","не указано, подписан ли документ второй стороной",IF(F8="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
+        <f>IF(COUNTA(B8:F8)=0,"",IF(OR(LEN(B8)=0,LEN(C8)=0,LEN(D8)=0,LEN(E8)=0,LEN(F8)=0),"НЕ ЗАПОЛНЕНО: основание, описание, сумма, документ и подпись",IF(NOT(OR(B8="материалы переданы генподрядчику",B8="материалы и оборудование остались на объекте",B8="затраты на мобилизацию и демобилизацию",B8="гарантийное удержание из оплаченных актов",B8="иное")),"ОШИБКА: неизвестное основание встречной суммы",IF(NOT(ISNUMBER(D8)),"ОШИБКА: сумма должна быть числом",IF(D8&lt;0,"ОШИБКА: отрицательная сумма",IF(AND(F8&lt;&gt;"да",F8&lt;&gt;"нет"),"ОШИБКА: подпись — выберите да или нет",IF(F8="нет","ПРОВЕРЬТЕ: самостоятельное основание и доказательства","строка заполнена")))))))</f>
+        <v/>
       </c>
     </row>
     <row r="9" ht="45" customHeight="1">
@@ -2308,7 +2381,8 @@
       <c r="E9" s="16" t="n"/>
       <c r="F9" s="16" t="n"/>
       <c r="G9" s="15">
-        <f>IF(D9="","",IF(B9="","не выбрано основание",IF(E9="","ОШИБКА: сумма без подтверждающего документа",IF(F9="","не указано, подписан ли документ второй стороной",IF(F9="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
+        <f>IF(COUNTA(B9:F9)=0,"",IF(OR(LEN(B9)=0,LEN(C9)=0,LEN(D9)=0,LEN(E9)=0,LEN(F9)=0),"НЕ ЗАПОЛНЕНО: основание, описание, сумма, документ и подпись",IF(NOT(OR(B9="материалы переданы генподрядчику",B9="материалы и оборудование остались на объекте",B9="затраты на мобилизацию и демобилизацию",B9="гарантийное удержание из оплаченных актов",B9="иное")),"ОШИБКА: неизвестное основание встречной суммы",IF(NOT(ISNUMBER(D9)),"ОШИБКА: сумма должна быть числом",IF(D9&lt;0,"ОШИБКА: отрицательная сумма",IF(AND(F9&lt;&gt;"да",F9&lt;&gt;"нет"),"ОШИБКА: подпись — выберите да или нет",IF(F9="нет","ПРОВЕРЬТЕ: самостоятельное основание и доказательства","строка заполнена")))))))</f>
+        <v/>
       </c>
     </row>
     <row r="10" ht="45" customHeight="1">
@@ -2322,7 +2396,8 @@
       <c r="E10" s="16" t="n"/>
       <c r="F10" s="16" t="n"/>
       <c r="G10" s="15">
-        <f>IF(D10="","",IF(B10="","не выбрано основание",IF(E10="","ОШИБКА: сумма без подтверждающего документа",IF(F10="","не указано, подписан ли документ второй стороной",IF(F10="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
+        <f>IF(COUNTA(B10:F10)=0,"",IF(OR(LEN(B10)=0,LEN(C10)=0,LEN(D10)=0,LEN(E10)=0,LEN(F10)=0),"НЕ ЗАПОЛНЕНО: основание, описание, сумма, документ и подпись",IF(NOT(OR(B10="материалы переданы генподрядчику",B10="материалы и оборудование остались на объекте",B10="затраты на мобилизацию и демобилизацию",B10="гарантийное удержание из оплаченных актов",B10="иное")),"ОШИБКА: неизвестное основание встречной суммы",IF(NOT(ISNUMBER(D10)),"ОШИБКА: сумма должна быть числом",IF(D10&lt;0,"ОШИБКА: отрицательная сумма",IF(AND(F10&lt;&gt;"да",F10&lt;&gt;"нет"),"ОШИБКА: подпись — выберите да или нет",IF(F10="нет","ПРОВЕРЬТЕ: самостоятельное основание и доказательства","строка заполнена")))))))</f>
+        <v/>
       </c>
     </row>
     <row r="11" ht="45" customHeight="1">
@@ -2336,7 +2411,8 @@
       <c r="E11" s="16" t="n"/>
       <c r="F11" s="16" t="n"/>
       <c r="G11" s="15">
-        <f>IF(D11="","",IF(B11="","не выбрано основание",IF(E11="","ОШИБКА: сумма без подтверждающего документа",IF(F11="","не указано, подписан ли документ второй стороной",IF(F11="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
+        <f>IF(COUNTA(B11:F11)=0,"",IF(OR(LEN(B11)=0,LEN(C11)=0,LEN(D11)=0,LEN(E11)=0,LEN(F11)=0),"НЕ ЗАПОЛНЕНО: основание, описание, сумма, документ и подпись",IF(NOT(OR(B11="материалы переданы генподрядчику",B11="материалы и оборудование остались на объекте",B11="затраты на мобилизацию и демобилизацию",B11="гарантийное удержание из оплаченных актов",B11="иное")),"ОШИБКА: неизвестное основание встречной суммы",IF(NOT(ISNUMBER(D11)),"ОШИБКА: сумма должна быть числом",IF(D11&lt;0,"ОШИБКА: отрицательная сумма",IF(AND(F11&lt;&gt;"да",F11&lt;&gt;"нет"),"ОШИБКА: подпись — выберите да или нет",IF(F11="нет","ПРОВЕРЬТЕ: самостоятельное основание и доказательства","строка заполнена")))))))</f>
+        <v/>
       </c>
     </row>
     <row r="12" ht="45" customHeight="1">
@@ -2350,7 +2426,8 @@
       <c r="E12" s="16" t="n"/>
       <c r="F12" s="16" t="n"/>
       <c r="G12" s="15">
-        <f>IF(D12="","",IF(B12="","не выбрано основание",IF(E12="","ОШИБКА: сумма без подтверждающего документа",IF(F12="","не указано, подписан ли документ второй стороной",IF(F12="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
+        <f>IF(COUNTA(B12:F12)=0,"",IF(OR(LEN(B12)=0,LEN(C12)=0,LEN(D12)=0,LEN(E12)=0,LEN(F12)=0),"НЕ ЗАПОЛНЕНО: основание, описание, сумма, документ и подпись",IF(NOT(OR(B12="материалы переданы генподрядчику",B12="материалы и оборудование остались на объекте",B12="затраты на мобилизацию и демобилизацию",B12="гарантийное удержание из оплаченных актов",B12="иное")),"ОШИБКА: неизвестное основание встречной суммы",IF(NOT(ISNUMBER(D12)),"ОШИБКА: сумма должна быть числом",IF(D12&lt;0,"ОШИБКА: отрицательная сумма",IF(AND(F12&lt;&gt;"да",F12&lt;&gt;"нет"),"ОШИБКА: подпись — выберите да или нет",IF(F12="нет","ПРОВЕРЬТЕ: самостоятельное основание и доказательства","строка заполнена")))))))</f>
+        <v/>
       </c>
     </row>
     <row r="13" ht="45" customHeight="1">
@@ -2364,7 +2441,8 @@
       <c r="E13" s="16" t="n"/>
       <c r="F13" s="16" t="n"/>
       <c r="G13" s="15">
-        <f>IF(D13="","",IF(B13="","не выбрано основание",IF(E13="","ОШИБКА: сумма без подтверждающего документа",IF(F13="","не указано, подписан ли документ второй стороной",IF(F13="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
+        <f>IF(COUNTA(B13:F13)=0,"",IF(OR(LEN(B13)=0,LEN(C13)=0,LEN(D13)=0,LEN(E13)=0,LEN(F13)=0),"НЕ ЗАПОЛНЕНО: основание, описание, сумма, документ и подпись",IF(NOT(OR(B13="материалы переданы генподрядчику",B13="материалы и оборудование остались на объекте",B13="затраты на мобилизацию и демобилизацию",B13="гарантийное удержание из оплаченных актов",B13="иное")),"ОШИБКА: неизвестное основание встречной суммы",IF(NOT(ISNUMBER(D13)),"ОШИБКА: сумма должна быть числом",IF(D13&lt;0,"ОШИБКА: отрицательная сумма",IF(AND(F13&lt;&gt;"да",F13&lt;&gt;"нет"),"ОШИБКА: подпись — выберите да или нет",IF(F13="нет","ПРОВЕРЬТЕ: самостоятельное основание и доказательства","строка заполнена")))))))</f>
+        <v/>
       </c>
     </row>
     <row r="14" ht="45" customHeight="1">
@@ -2378,7 +2456,8 @@
       <c r="E14" s="16" t="n"/>
       <c r="F14" s="16" t="n"/>
       <c r="G14" s="15">
-        <f>IF(D14="","",IF(B14="","не выбрано основание",IF(E14="","ОШИБКА: сумма без подтверждающего документа",IF(F14="","не указано, подписан ли документ второй стороной",IF(F14="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
+        <f>IF(COUNTA(B14:F14)=0,"",IF(OR(LEN(B14)=0,LEN(C14)=0,LEN(D14)=0,LEN(E14)=0,LEN(F14)=0),"НЕ ЗАПОЛНЕНО: основание, описание, сумма, документ и подпись",IF(NOT(OR(B14="материалы переданы генподрядчику",B14="материалы и оборудование остались на объекте",B14="затраты на мобилизацию и демобилизацию",B14="гарантийное удержание из оплаченных актов",B14="иное")),"ОШИБКА: неизвестное основание встречной суммы",IF(NOT(ISNUMBER(D14)),"ОШИБКА: сумма должна быть числом",IF(D14&lt;0,"ОШИБКА: отрицательная сумма",IF(AND(F14&lt;&gt;"да",F14&lt;&gt;"нет"),"ОШИБКА: подпись — выберите да или нет",IF(F14="нет","ПРОВЕРЬТЕ: самостоятельное основание и доказательства","строка заполнена")))))))</f>
+        <v/>
       </c>
     </row>
     <row r="15" ht="45" customHeight="1">
@@ -2392,7 +2471,8 @@
       <c r="E15" s="16" t="n"/>
       <c r="F15" s="16" t="n"/>
       <c r="G15" s="15">
-        <f>IF(D15="","",IF(B15="","не выбрано основание",IF(E15="","ОШИБКА: сумма без подтверждающего документа",IF(F15="","не указано, подписан ли документ второй стороной",IF(F15="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
+        <f>IF(COUNTA(B15:F15)=0,"",IF(OR(LEN(B15)=0,LEN(C15)=0,LEN(D15)=0,LEN(E15)=0,LEN(F15)=0),"НЕ ЗАПОЛНЕНО: основание, описание, сумма, документ и подпись",IF(NOT(OR(B15="материалы переданы генподрядчику",B15="материалы и оборудование остались на объекте",B15="затраты на мобилизацию и демобилизацию",B15="гарантийное удержание из оплаченных актов",B15="иное")),"ОШИБКА: неизвестное основание встречной суммы",IF(NOT(ISNUMBER(D15)),"ОШИБКА: сумма должна быть числом",IF(D15&lt;0,"ОШИБКА: отрицательная сумма",IF(AND(F15&lt;&gt;"да",F15&lt;&gt;"нет"),"ОШИБКА: подпись — выберите да или нет",IF(F15="нет","ПРОВЕРЬТЕ: самостоятельное основание и доказательства","строка заполнена")))))))</f>
+        <v/>
       </c>
     </row>
     <row r="16" ht="45" customHeight="1">
@@ -2406,7 +2486,8 @@
       <c r="E16" s="16" t="n"/>
       <c r="F16" s="16" t="n"/>
       <c r="G16" s="15">
-        <f>IF(D16="","",IF(B16="","не выбрано основание",IF(E16="","ОШИБКА: сумма без подтверждающего документа",IF(F16="","не указано, подписан ли документ второй стороной",IF(F16="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
+        <f>IF(COUNTA(B16:F16)=0,"",IF(OR(LEN(B16)=0,LEN(C16)=0,LEN(D16)=0,LEN(E16)=0,LEN(F16)=0),"НЕ ЗАПОЛНЕНО: основание, описание, сумма, документ и подпись",IF(NOT(OR(B16="материалы переданы генподрядчику",B16="материалы и оборудование остались на объекте",B16="затраты на мобилизацию и демобилизацию",B16="гарантийное удержание из оплаченных актов",B16="иное")),"ОШИБКА: неизвестное основание встречной суммы",IF(NOT(ISNUMBER(D16)),"ОШИБКА: сумма должна быть числом",IF(D16&lt;0,"ОШИБКА: отрицательная сумма",IF(AND(F16&lt;&gt;"да",F16&lt;&gt;"нет"),"ОШИБКА: подпись — выберите да или нет",IF(F16="нет","ПРОВЕРЬТЕ: самостоятельное основание и доказательства","строка заполнена")))))))</f>
+        <v/>
       </c>
     </row>
     <row r="17" ht="45" customHeight="1">
@@ -2420,7 +2501,8 @@
       <c r="E17" s="16" t="n"/>
       <c r="F17" s="16" t="n"/>
       <c r="G17" s="15">
-        <f>IF(D17="","",IF(B17="","не выбрано основание",IF(E17="","ОШИБКА: сумма без подтверждающего документа",IF(F17="","не указано, подписан ли документ второй стороной",IF(F17="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
+        <f>IF(COUNTA(B17:F17)=0,"",IF(OR(LEN(B17)=0,LEN(C17)=0,LEN(D17)=0,LEN(E17)=0,LEN(F17)=0),"НЕ ЗАПОЛНЕНО: основание, описание, сумма, документ и подпись",IF(NOT(OR(B17="материалы переданы генподрядчику",B17="материалы и оборудование остались на объекте",B17="затраты на мобилизацию и демобилизацию",B17="гарантийное удержание из оплаченных актов",B17="иное")),"ОШИБКА: неизвестное основание встречной суммы",IF(NOT(ISNUMBER(D17)),"ОШИБКА: сумма должна быть числом",IF(D17&lt;0,"ОШИБКА: отрицательная сумма",IF(AND(F17&lt;&gt;"да",F17&lt;&gt;"нет"),"ОШИБКА: подпись — выберите да или нет",IF(F17="нет","ПРОВЕРЬТЕ: самостоятельное основание и доказательства","строка заполнена")))))))</f>
+        <v/>
       </c>
     </row>
     <row r="18" ht="45" customHeight="1">
@@ -2434,7 +2516,8 @@
       <c r="E18" s="16" t="n"/>
       <c r="F18" s="16" t="n"/>
       <c r="G18" s="15">
-        <f>IF(D18="","",IF(B18="","не выбрано основание",IF(E18="","ОШИБКА: сумма без подтверждающего документа",IF(F18="","не указано, подписан ли документ второй стороной",IF(F18="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
+        <f>IF(COUNTA(B18:F18)=0,"",IF(OR(LEN(B18)=0,LEN(C18)=0,LEN(D18)=0,LEN(E18)=0,LEN(F18)=0),"НЕ ЗАПОЛНЕНО: основание, описание, сумма, документ и подпись",IF(NOT(OR(B18="материалы переданы генподрядчику",B18="материалы и оборудование остались на объекте",B18="затраты на мобилизацию и демобилизацию",B18="гарантийное удержание из оплаченных актов",B18="иное")),"ОШИБКА: неизвестное основание встречной суммы",IF(NOT(ISNUMBER(D18)),"ОШИБКА: сумма должна быть числом",IF(D18&lt;0,"ОШИБКА: отрицательная сумма",IF(AND(F18&lt;&gt;"да",F18&lt;&gt;"нет"),"ОШИБКА: подпись — выберите да или нет",IF(F18="нет","ПРОВЕРЬТЕ: самостоятельное основание и доказательства","строка заполнена")))))))</f>
+        <v/>
       </c>
     </row>
     <row r="19" ht="45" customHeight="1">
@@ -2448,7 +2531,8 @@
       <c r="E19" s="16" t="n"/>
       <c r="F19" s="16" t="n"/>
       <c r="G19" s="15">
-        <f>IF(D19="","",IF(B19="","не выбрано основание",IF(E19="","ОШИБКА: сумма без подтверждающего документа",IF(F19="","не указано, подписан ли документ второй стороной",IF(F19="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
+        <f>IF(COUNTA(B19:F19)=0,"",IF(OR(LEN(B19)=0,LEN(C19)=0,LEN(D19)=0,LEN(E19)=0,LEN(F19)=0),"НЕ ЗАПОЛНЕНО: основание, описание, сумма, документ и подпись",IF(NOT(OR(B19="материалы переданы генподрядчику",B19="материалы и оборудование остались на объекте",B19="затраты на мобилизацию и демобилизацию",B19="гарантийное удержание из оплаченных актов",B19="иное")),"ОШИБКА: неизвестное основание встречной суммы",IF(NOT(ISNUMBER(D19)),"ОШИБКА: сумма должна быть числом",IF(D19&lt;0,"ОШИБКА: отрицательная сумма",IF(AND(F19&lt;&gt;"да",F19&lt;&gt;"нет"),"ОШИБКА: подпись — выберите да или нет",IF(F19="нет","ПРОВЕРЬТЕ: самостоятельное основание и доказательства","строка заполнена")))))))</f>
+        <v/>
       </c>
     </row>
     <row r="20" ht="45" customHeight="1">
@@ -2462,7 +2546,8 @@
       <c r="E20" s="16" t="n"/>
       <c r="F20" s="16" t="n"/>
       <c r="G20" s="15">
-        <f>IF(D20="","",IF(B20="","не выбрано основание",IF(E20="","ОШИБКА: сумма без подтверждающего документа",IF(F20="","не указано, подписан ли документ второй стороной",IF(F20="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
+        <f>IF(COUNTA(B20:F20)=0,"",IF(OR(LEN(B20)=0,LEN(C20)=0,LEN(D20)=0,LEN(E20)=0,LEN(F20)=0),"НЕ ЗАПОЛНЕНО: основание, описание, сумма, документ и подпись",IF(NOT(OR(B20="материалы переданы генподрядчику",B20="материалы и оборудование остались на объекте",B20="затраты на мобилизацию и демобилизацию",B20="гарантийное удержание из оплаченных актов",B20="иное")),"ОШИБКА: неизвестное основание встречной суммы",IF(NOT(ISNUMBER(D20)),"ОШИБКА: сумма должна быть числом",IF(D20&lt;0,"ОШИБКА: отрицательная сумма",IF(AND(F20&lt;&gt;"да",F20&lt;&gt;"нет"),"ОШИБКА: подпись — выберите да или нет",IF(F20="нет","ПРОВЕРЬТЕ: самостоятельное основание и доказательства","строка заполнена")))))))</f>
+        <v/>
       </c>
     </row>
     <row r="21" ht="45" customHeight="1">
@@ -2476,7 +2561,8 @@
       <c r="E21" s="16" t="n"/>
       <c r="F21" s="16" t="n"/>
       <c r="G21" s="15">
-        <f>IF(D21="","",IF(B21="","не выбрано основание",IF(E21="","ОШИБКА: сумма без подтверждающего документа",IF(F21="","не указано, подписан ли документ второй стороной",IF(F21="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
+        <f>IF(COUNTA(B21:F21)=0,"",IF(OR(LEN(B21)=0,LEN(C21)=0,LEN(D21)=0,LEN(E21)=0,LEN(F21)=0),"НЕ ЗАПОЛНЕНО: основание, описание, сумма, документ и подпись",IF(NOT(OR(B21="материалы переданы генподрядчику",B21="материалы и оборудование остались на объекте",B21="затраты на мобилизацию и демобилизацию",B21="гарантийное удержание из оплаченных актов",B21="иное")),"ОШИБКА: неизвестное основание встречной суммы",IF(NOT(ISNUMBER(D21)),"ОШИБКА: сумма должна быть числом",IF(D21&lt;0,"ОШИБКА: отрицательная сумма",IF(AND(F21&lt;&gt;"да",F21&lt;&gt;"нет"),"ОШИБКА: подпись — выберите да или нет",IF(F21="нет","ПРОВЕРЬТЕ: самостоятельное основание и доказательства","строка заполнена")))))))</f>
+        <v/>
       </c>
     </row>
     <row r="22" ht="45" customHeight="1">
@@ -2490,7 +2576,8 @@
       <c r="E22" s="16" t="n"/>
       <c r="F22" s="16" t="n"/>
       <c r="G22" s="15">
-        <f>IF(D22="","",IF(B22="","не выбрано основание",IF(E22="","ОШИБКА: сумма без подтверждающего документа",IF(F22="","не указано, подписан ли документ второй стороной",IF(F22="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
+        <f>IF(COUNTA(B22:F22)=0,"",IF(OR(LEN(B22)=0,LEN(C22)=0,LEN(D22)=0,LEN(E22)=0,LEN(F22)=0),"НЕ ЗАПОЛНЕНО: основание, описание, сумма, документ и подпись",IF(NOT(OR(B22="материалы переданы генподрядчику",B22="материалы и оборудование остались на объекте",B22="затраты на мобилизацию и демобилизацию",B22="гарантийное удержание из оплаченных актов",B22="иное")),"ОШИБКА: неизвестное основание встречной суммы",IF(NOT(ISNUMBER(D22)),"ОШИБКА: сумма должна быть числом",IF(D22&lt;0,"ОШИБКА: отрицательная сумма",IF(AND(F22&lt;&gt;"да",F22&lt;&gt;"нет"),"ОШИБКА: подпись — выберите да или нет",IF(F22="нет","ПРОВЕРЬТЕ: самостоятельное основание и доказательства","строка заполнена")))))))</f>
+        <v/>
       </c>
     </row>
     <row r="23" ht="45" customHeight="1">
@@ -2504,7 +2591,8 @@
       <c r="E23" s="16" t="n"/>
       <c r="F23" s="16" t="n"/>
       <c r="G23" s="15">
-        <f>IF(D23="","",IF(B23="","не выбрано основание",IF(E23="","ОШИБКА: сумма без подтверждающего документа",IF(F23="","не указано, подписан ли документ второй стороной",IF(F23="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
+        <f>IF(COUNTA(B23:F23)=0,"",IF(OR(LEN(B23)=0,LEN(C23)=0,LEN(D23)=0,LEN(E23)=0,LEN(F23)=0),"НЕ ЗАПОЛНЕНО: основание, описание, сумма, документ и подпись",IF(NOT(OR(B23="материалы переданы генподрядчику",B23="материалы и оборудование остались на объекте",B23="затраты на мобилизацию и демобилизацию",B23="гарантийное удержание из оплаченных актов",B23="иное")),"ОШИБКА: неизвестное основание встречной суммы",IF(NOT(ISNUMBER(D23)),"ОШИБКА: сумма должна быть числом",IF(D23&lt;0,"ОШИБКА: отрицательная сумма",IF(AND(F23&lt;&gt;"да",F23&lt;&gt;"нет"),"ОШИБКА: подпись — выберите да или нет",IF(F23="нет","ПРОВЕРЬТЕ: самостоятельное основание и доказательства","строка заполнена")))))))</f>
+        <v/>
       </c>
     </row>
     <row r="24" ht="45" customHeight="1">
@@ -2518,7 +2606,8 @@
       <c r="E24" s="16" t="n"/>
       <c r="F24" s="16" t="n"/>
       <c r="G24" s="15">
-        <f>IF(D24="","",IF(B24="","не выбрано основание",IF(E24="","ОШИБКА: сумма без подтверждающего документа",IF(F24="","не указано, подписан ли документ второй стороной",IF(F24="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
+        <f>IF(COUNTA(B24:F24)=0,"",IF(OR(LEN(B24)=0,LEN(C24)=0,LEN(D24)=0,LEN(E24)=0,LEN(F24)=0),"НЕ ЗАПОЛНЕНО: основание, описание, сумма, документ и подпись",IF(NOT(OR(B24="материалы переданы генподрядчику",B24="материалы и оборудование остались на объекте",B24="затраты на мобилизацию и демобилизацию",B24="гарантийное удержание из оплаченных актов",B24="иное")),"ОШИБКА: неизвестное основание встречной суммы",IF(NOT(ISNUMBER(D24)),"ОШИБКА: сумма должна быть числом",IF(D24&lt;0,"ОШИБКА: отрицательная сумма",IF(AND(F24&lt;&gt;"да",F24&lt;&gt;"нет"),"ОШИБКА: подпись — выберите да или нет",IF(F24="нет","ПРОВЕРЬТЕ: самостоятельное основание и доказательства","строка заполнена")))))))</f>
+        <v/>
       </c>
     </row>
     <row r="25" ht="45" customHeight="1">
@@ -2532,7 +2621,8 @@
       <c r="E25" s="16" t="n"/>
       <c r="F25" s="16" t="n"/>
       <c r="G25" s="15">
-        <f>IF(D25="","",IF(B25="","не выбрано основание",IF(E25="","ОШИБКА: сумма без подтверждающего документа",IF(F25="","не указано, подписан ли документ второй стороной",IF(F25="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
+        <f>IF(COUNTA(B25:F25)=0,"",IF(OR(LEN(B25)=0,LEN(C25)=0,LEN(D25)=0,LEN(E25)=0,LEN(F25)=0),"НЕ ЗАПОЛНЕНО: основание, описание, сумма, документ и подпись",IF(NOT(OR(B25="материалы переданы генподрядчику",B25="материалы и оборудование остались на объекте",B25="затраты на мобилизацию и демобилизацию",B25="гарантийное удержание из оплаченных актов",B25="иное")),"ОШИБКА: неизвестное основание встречной суммы",IF(NOT(ISNUMBER(D25)),"ОШИБКА: сумма должна быть числом",IF(D25&lt;0,"ОШИБКА: отрицательная сумма",IF(AND(F25&lt;&gt;"да",F25&lt;&gt;"нет"),"ОШИБКА: подпись — выберите да или нет",IF(F25="нет","ПРОВЕРЬТЕ: самостоятельное основание и доказательства","строка заполнена")))))))</f>
+        <v/>
       </c>
     </row>
     <row r="26" ht="45" customHeight="1">
@@ -2546,7 +2636,8 @@
       <c r="E26" s="16" t="n"/>
       <c r="F26" s="16" t="n"/>
       <c r="G26" s="15">
-        <f>IF(D26="","",IF(B26="","не выбрано основание",IF(E26="","ОШИБКА: сумма без подтверждающего документа",IF(F26="","не указано, подписан ли документ второй стороной",IF(F26="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
+        <f>IF(COUNTA(B26:F26)=0,"",IF(OR(LEN(B26)=0,LEN(C26)=0,LEN(D26)=0,LEN(E26)=0,LEN(F26)=0),"НЕ ЗАПОЛНЕНО: основание, описание, сумма, документ и подпись",IF(NOT(OR(B26="материалы переданы генподрядчику",B26="материалы и оборудование остались на объекте",B26="затраты на мобилизацию и демобилизацию",B26="гарантийное удержание из оплаченных актов",B26="иное")),"ОШИБКА: неизвестное основание встречной суммы",IF(NOT(ISNUMBER(D26)),"ОШИБКА: сумма должна быть числом",IF(D26&lt;0,"ОШИБКА: отрицательная сумма",IF(AND(F26&lt;&gt;"да",F26&lt;&gt;"нет"),"ОШИБКА: подпись — выберите да или нет",IF(F26="нет","ПРОВЕРЬТЕ: самостоятельное основание и доказательства","строка заполнена")))))))</f>
+        <v/>
       </c>
     </row>
     <row r="27" ht="45" customHeight="1">
@@ -2560,7 +2651,8 @@
       <c r="E27" s="16" t="n"/>
       <c r="F27" s="16" t="n"/>
       <c r="G27" s="15">
-        <f>IF(D27="","",IF(B27="","не выбрано основание",IF(E27="","ОШИБКА: сумма без подтверждающего документа",IF(F27="","не указано, подписан ли документ второй стороной",IF(F27="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
+        <f>IF(COUNTA(B27:F27)=0,"",IF(OR(LEN(B27)=0,LEN(C27)=0,LEN(D27)=0,LEN(E27)=0,LEN(F27)=0),"НЕ ЗАПОЛНЕНО: основание, описание, сумма, документ и подпись",IF(NOT(OR(B27="материалы переданы генподрядчику",B27="материалы и оборудование остались на объекте",B27="затраты на мобилизацию и демобилизацию",B27="гарантийное удержание из оплаченных актов",B27="иное")),"ОШИБКА: неизвестное основание встречной суммы",IF(NOT(ISNUMBER(D27)),"ОШИБКА: сумма должна быть числом",IF(D27&lt;0,"ОШИБКА: отрицательная сумма",IF(AND(F27&lt;&gt;"да",F27&lt;&gt;"нет"),"ОШИБКА: подпись — выберите да или нет",IF(F27="нет","ПРОВЕРЬТЕ: самостоятельное основание и доказательства","строка заполнена")))))))</f>
+        <v/>
       </c>
     </row>
     <row r="28" ht="45" customHeight="1">
@@ -2574,7 +2666,8 @@
       <c r="E28" s="16" t="n"/>
       <c r="F28" s="16" t="n"/>
       <c r="G28" s="15">
-        <f>IF(D28="","",IF(B28="","не выбрано основание",IF(E28="","ОШИБКА: сумма без подтверждающего документа",IF(F28="","не указано, подписан ли документ второй стороной",IF(F28="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
+        <f>IF(COUNTA(B28:F28)=0,"",IF(OR(LEN(B28)=0,LEN(C28)=0,LEN(D28)=0,LEN(E28)=0,LEN(F28)=0),"НЕ ЗАПОЛНЕНО: основание, описание, сумма, документ и подпись",IF(NOT(OR(B28="материалы переданы генподрядчику",B28="материалы и оборудование остались на объекте",B28="затраты на мобилизацию и демобилизацию",B28="гарантийное удержание из оплаченных актов",B28="иное")),"ОШИБКА: неизвестное основание встречной суммы",IF(NOT(ISNUMBER(D28)),"ОШИБКА: сумма должна быть числом",IF(D28&lt;0,"ОШИБКА: отрицательная сумма",IF(AND(F28&lt;&gt;"да",F28&lt;&gt;"нет"),"ОШИБКА: подпись — выберите да или нет",IF(F28="нет","ПРОВЕРЬТЕ: самостоятельное основание и доказательства","строка заполнена")))))))</f>
+        <v/>
       </c>
     </row>
     <row r="29" ht="45" customHeight="1">
@@ -2588,7 +2681,8 @@
       <c r="E29" s="16" t="n"/>
       <c r="F29" s="16" t="n"/>
       <c r="G29" s="15">
-        <f>IF(D29="","",IF(B29="","не выбрано основание",IF(E29="","ОШИБКА: сумма без подтверждающего документа",IF(F29="","не указано, подписан ли документ второй стороной",IF(F29="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
+        <f>IF(COUNTA(B29:F29)=0,"",IF(OR(LEN(B29)=0,LEN(C29)=0,LEN(D29)=0,LEN(E29)=0,LEN(F29)=0),"НЕ ЗАПОЛНЕНО: основание, описание, сумма, документ и подпись",IF(NOT(OR(B29="материалы переданы генподрядчику",B29="материалы и оборудование остались на объекте",B29="затраты на мобилизацию и демобилизацию",B29="гарантийное удержание из оплаченных актов",B29="иное")),"ОШИБКА: неизвестное основание встречной суммы",IF(NOT(ISNUMBER(D29)),"ОШИБКА: сумма должна быть числом",IF(D29&lt;0,"ОШИБКА: отрицательная сумма",IF(AND(F29&lt;&gt;"да",F29&lt;&gt;"нет"),"ОШИБКА: подпись — выберите да или нет",IF(F29="нет","ПРОВЕРЬТЕ: самостоятельное основание и доказательства","строка заполнена")))))))</f>
+        <v/>
       </c>
     </row>
     <row r="30" ht="45" customHeight="1">
@@ -2602,7 +2696,8 @@
       <c r="E30" s="16" t="n"/>
       <c r="F30" s="16" t="n"/>
       <c r="G30" s="15">
-        <f>IF(D30="","",IF(B30="","не выбрано основание",IF(E30="","ОШИБКА: сумма без подтверждающего документа",IF(F30="","не указано, подписан ли документ второй стороной",IF(F30="нет","Проверьте самостоятельное основание требования и подтверждающие документы.","строка заполнена")))))</f>
+        <f>IF(COUNTA(B30:F30)=0,"",IF(OR(LEN(B30)=0,LEN(C30)=0,LEN(D30)=0,LEN(E30)=0,LEN(F30)=0),"НЕ ЗАПОЛНЕНО: основание, описание, сумма, документ и подпись",IF(NOT(OR(B30="материалы переданы генподрядчику",B30="материалы и оборудование остались на объекте",B30="затраты на мобилизацию и демобилизацию",B30="гарантийное удержание из оплаченных актов",B30="иное")),"ОШИБКА: неизвестное основание встречной суммы",IF(NOT(ISNUMBER(D30)),"ОШИБКА: сумма должна быть числом",IF(D30&lt;0,"ОШИБКА: отрицательная сумма",IF(AND(F30&lt;&gt;"да",F30&lt;&gt;"нет"),"ОШИБКА: подпись — выберите да или нет",IF(F30="нет","ПРОВЕРЬТЕ: самостоятельное основание и доказательства","строка заполнена")))))))</f>
+        <v/>
       </c>
     </row>
     <row r="31">
@@ -2681,11 +2776,11 @@
     <row r="38">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>Строк с ошибкой в колонке «Проверка»</t>
+          <t>Строк с ошибками или незаполненными данными</t>
         </is>
       </c>
       <c r="D38" s="21">
-        <f>COUNTIF(G6:G30,"ОШИБКА*")</f>
+        <f>SUMPRODUCT(--(LEFT(G6:G30,6)="ОШИБКА"))+SUMPRODUCT(--(LEFT(G6:G30,12)="НЕ ЗАПОЛНЕНО"))</f>
         <v/>
       </c>
     </row>
@@ -2719,10 +2814,10 @@
     <mergeCell ref="A38:C38"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="B6:B30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="Выберите основание из списка" type="list">
+    <dataValidation type="list" errorStyle="stop" allowBlank="0" showDropDown="0" showErrorMessage="1" errorTitle="Проверка ввода" error="Выберите основание встречной суммы." sqref="B6:B30">
       <formula1>"материалы переданы генподрядчику,материалы и оборудование остались на объекте,затраты на мобилизацию и демобилизацию,гарантийное удержание из оплаченных актов,иное"</formula1>
     </dataValidation>
-    <dataValidation sqref="F6:F30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation type="list" errorStyle="stop" allowBlank="0" showDropDown="0" showErrorMessage="1" errorTitle="Проверка ввода" error="Выберите да или нет." sqref="F6:F30">
       <formula1>"да,нет"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2759,7 +2854,7 @@
     <row r="3" ht="26" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">До использования итогового сальдо проверьте сообщения раздела «Проверки» и устраните выявленные расхождения.</t>
+          <t>Если расчёт не завершён, итог не выводится. Исправьте ошибки и пустые обязательные поля. Правовое основание каждой заявляемой суммы проверяйте отдельно.</t>
         </is>
       </c>
     </row>
@@ -2809,7 +2904,7 @@
         </is>
       </c>
       <c r="B8" s="23">
-        <f>ROUND(B6+B7,2)</f>
+        <f>IF(AND(ISNUMBER(B6),ISNUMBER(B7)),ROUND(B6+B7,2),"")</f>
         <v/>
       </c>
       <c r="C8" s="4" t="inlineStr"/>
@@ -2910,32 +3005,32 @@
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Работы переданы, акты не подписаны</t>
+          <t>Неоплаченный остаток: акты переданы, не подписаны</t>
         </is>
       </c>
       <c r="B20" s="8">
-        <f>SUMIF('Выполнено'!F6:F45,"передан, не подписан",'Выполнено'!E6:E45)</f>
+        <f>SUMIF('Выполнено'!F6:F45,"передан, не подписан",'Выполнено'!K6:K45)</f>
         <v/>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Проверьте фактический объём, направление актов и доказательства получения.</t>
+          <t>Стоимость за вычетом отнесённой денежной оплаты. Проверьте объём, передачу и основание требования.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="60" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Работы переданы, акты подписаны односторонне</t>
+          <t>Неоплаченный остаток: односторонние акты</t>
         </is>
       </c>
       <c r="B21" s="8">
-        <f>SUMIF('Выполнено'!F6:F45,"подписан односторонне",'Выполнено'!E6:E45)</f>
+        <f>SUMIF('Выполнено'!F6:F45,"подписан односторонне",'Выполнено'!K6:K45)</f>
         <v/>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Проверьте оформление по пункту 4 статьи 753 ГК РФ, извещение, отметку об отказе и основания возражений.</t>
+          <t>Стоимость за вычетом отнесённой денежной оплаты. Статус акта и основания по п. 4 ст. 753 ГК РФ проверяются отдельно.</t>
         </is>
       </c>
     </row>
@@ -3069,7 +3164,7 @@
         </is>
       </c>
       <c r="B32" s="23">
-        <f>ROUND(B17-B27,2)</f>
+        <f>IF('Договор и аванс'!B19&lt;&gt;"заполнено","",IF(OR('Выполнено'!E55&gt;0,'Встречное'!D38&gt;0,B12&gt;B6+0.01,B37&lt;&gt;"Расхождений не выявлено"),"",ROUND(B17-B27,2)))</f>
         <v/>
       </c>
       <c r="C32" s="4" t="inlineStr">
@@ -3085,7 +3180,8 @@
         </is>
       </c>
       <c r="B33" s="24">
-        <f>IF(B32&gt;0,"к возврату генподрядчику",IF(B32&lt;0,"К оплате Субподрядчику","ноль"))</f>
+        <f>IF(NOT(ISNUMBER(B32)),"Расчёт не завершён",IF(B32&gt;0,"к возврату генподрядчику",IF(B32&lt;0,"К оплате Субподрядчику","ноль")))</f>
+        <v/>
       </c>
       <c r="C33" s="4" t="inlineStr"/>
     </row>
@@ -3096,7 +3192,7 @@
         </is>
       </c>
       <c r="B34" s="8">
-        <f>ROUND(B30-B31,2)</f>
+        <f>IF(AND(ISNUMBER(B30),ISNUMBER(B31)),ROUND(B30-B31,2),"")</f>
         <v/>
       </c>
       <c r="C34" s="4" t="inlineStr">
@@ -3119,11 +3215,12 @@
         </is>
       </c>
       <c r="B37" s="25">
-        <f>IF(ROUND(B11-B8,2)=ROUND(B14-B17,2),"Расхождений не выявлено","ПРОВЕРЬТЕ: платежи отнесены к актам, не подписанным обеими сторонами; расхождение "&amp;ROUND((B11-B8)-(B14-B17),2))</f>
+        <f>IFERROR(IF(ABS(ROUND(B6+B7-B11-SUMIF('Выполнено'!F6:F45,"передан, не подписан",'Выполнено'!E6:E45)-SUMIF('Выполнено'!F6:F45,"подписан односторонне",'Выполнено'!E6:E45)-SUM(B22:B25),2)-ROUND(B17-B27,2))&lt;0.01,"Расхождений не выявлено","ПРОВЕРЬТЕ: отнесение оплат и погашение аванса"),"ПРОВЕРЬТЕ: числовые исходные данные")</f>
+        <v/>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Сопоставьте поступления и стоимость принятых работ с расчётом от аванса. При расхождении проверьте отнесение каждого платежа к соответствующему акту.</t>
+          <t>Сверка поступлений, стоимости включённых актов и встречных сумм. Платежи по исключённым актам и погашение сверх аванса требуют разбора.</t>
         </is>
       </c>
     </row>
@@ -3134,7 +3231,7 @@
         </is>
       </c>
       <c r="B38" s="25">
-        <f>IF(COUNTIF('Выполнено'!L6:L45,"ОШИБКА*")=0,"нет","ПРОВЕРЬТЕ: строк с ошибкой — "&amp;COUNTIF('Выполнено'!L6:L45,"ОШИБКА*"))</f>
+        <f>IF('Выполнено'!E55=0,"нет","ПРОВЕРЬТЕ: незавершённых/ошибочных строк — "&amp;'Выполнено'!E55)</f>
         <v/>
       </c>
       <c r="C38" s="4" t="inlineStr">
@@ -3150,7 +3247,7 @@
         </is>
       </c>
       <c r="B39" s="25">
-        <f>IF(COUNTIF('Встречное'!G6:G30,"ОШИБКА*")=0,"нет","ПРОВЕРЬТЕ: сумм без подтверждающего документа — "&amp;COUNTIF('Встречное'!G6:G30,"ОШИБКА*"))</f>
+        <f>IF('Встречное'!D38=0,"нет","ПРОВЕРЬТЕ: незавершённых/ошибочных строк — "&amp;'Встречное'!D38)</f>
         <v/>
       </c>
       <c r="C39" s="4" t="inlineStr">
@@ -3414,7 +3511,7 @@
         </is>
       </c>
       <c r="B16" s="23">
-        <f>ROUND(B15-C15,2)</f>
+        <f>IF(NOT(ISNUMBER('Сальдо'!B32)),"",ROUND(B15-C15,2))</f>
         <v/>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -3425,11 +3522,11 @@
     </row>
     <row r="18" ht="32" customHeight="1">
       <c r="A18" s="3">
-        <f>IF(B16&lt;0,"По данным Субподрядчика на указанную дату за Субподрядчиком числится задолженность в размере, руб.:","По данным Субподрядчика на указанную дату за Генподрядчиком числится задолженность в размере, руб.:")</f>
+        <f>IF(NOT(ISNUMBER(B16)),"Расчёт не завершён: проверьте исходные данные",IF(B16&lt;0,"По данным Субподрядчика на указанную дату за Субподрядчиком числится задолженность в размере, руб.:","По данным Субподрядчика на указанную дату за Генподрядчиком числится задолженность в размере, руб.:"))</f>
         <v/>
       </c>
       <c r="D18" s="23">
-        <f>ROUND(MAX(B16,-B16),2)</f>
+        <f>IF(NOT(ISNUMBER(B16)),"",ROUND(MAX(B16,-B16),2))</f>
         <v/>
       </c>
     </row>

</xml_diff>